<commit_message>
feat: Implement comprehensive deal and portfolio analysis features including IC memo, track record, and methodology views with supporting metrics, models, and UI updates.
</commit_message>
<xml_diff>
--- a/PE_Fund_Data_Template.xlsx
+++ b/PE_Fund_Data_Template.xlsx
@@ -7,7 +7,11 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deals" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cashflows" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deal Quarterly" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fund Quarterly" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Underwrite" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,8 +21,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
+    <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="2">
     <font>
@@ -58,11 +62,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -429,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U13"/>
+  <dimension ref="A1:AD13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -460,82 +466,127 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>Exit Type</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Lead Partner</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Security Type</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Deal Type</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Entry Channel</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
           <t>Investment Date</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Year Invested</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Exit Date</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Equity Invested</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Ownership %</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Entry Revenue</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Entry EBITDA</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Entry EV</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Entry Net Debt</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Exit Revenue</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Exit EBITDA</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>Exit EV</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>Exit Net Debt</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>Realized Value</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>Unrealized Value</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>IRR</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
+        <is>
+          <t>Fund Size</t>
+        </is>
+      </c>
+      <c r="AB1" t="inlineStr">
+        <is>
+          <t>Net IRR</t>
+        </is>
+      </c>
+      <c r="AC1" t="inlineStr">
+        <is>
+          <t>Net MOIC</t>
+        </is>
+      </c>
+      <c r="AD1" t="inlineStr">
+        <is>
+          <t>DPI</t>
         </is>
       </c>
     </row>
@@ -557,7 +608,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>US</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -565,51 +616,90 @@
           <t>Fully Realized</t>
         </is>
       </c>
-      <c r="F2" s="2" t="n">
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>Strategic Sale</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>A. Morgan</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>Common Equity</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Platform</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Proprietary</t>
+        </is>
+      </c>
+      <c r="K2" s="4" t="n">
         <v>43174</v>
       </c>
-      <c r="G2" t="n">
+      <c r="L2" t="n">
         <v>2018</v>
       </c>
-      <c r="H2" s="2" t="n">
+      <c r="M2" s="4" t="n">
         <v>45107</v>
       </c>
-      <c r="I2" t="n">
+      <c r="N2" t="n">
         <v>75</v>
       </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="n">
+      <c r="O2" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="P2" t="n">
         <v>120</v>
       </c>
-      <c r="L2" t="n">
+      <c r="Q2" t="n">
         <v>28</v>
       </c>
-      <c r="M2" t="n">
+      <c r="R2" t="n">
         <v>310</v>
       </c>
-      <c r="N2" t="n">
+      <c r="S2" t="n">
         <v>85</v>
       </c>
-      <c r="O2" t="n">
+      <c r="T2" t="n">
         <v>245</v>
       </c>
-      <c r="P2" t="n">
+      <c r="U2" t="n">
         <v>62</v>
       </c>
-      <c r="Q2" t="n">
+      <c r="V2" t="n">
         <v>720</v>
       </c>
-      <c r="R2" t="n">
+      <c r="W2" t="n">
         <v>95</v>
       </c>
-      <c r="S2" t="n">
+      <c r="X2" t="n">
+        <v>170</v>
+      </c>
+      <c r="Y2" t="n">
         <v>0</v>
       </c>
-      <c r="T2" t="n">
-        <v>0</v>
-      </c>
-      <c r="U2" t="n">
+      <c r="Z2" t="n">
         <v>0.28</v>
+      </c>
+      <c r="AA2" t="n">
+        <v>620</v>
+      </c>
+      <c r="AB2" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="AC2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AD2" t="n">
+        <v>1.4</v>
       </c>
     </row>
     <row r="3">
@@ -630,7 +720,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>US</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -638,51 +728,90 @@
           <t>Fully Realized</t>
         </is>
       </c>
-      <c r="F3" s="2" t="n">
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Secondary Buyout</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>L. Chen</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Preferred Equity</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Platform</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Limited Auction</t>
+        </is>
+      </c>
+      <c r="K3" s="4" t="n">
         <v>43475</v>
       </c>
-      <c r="G3" t="n">
+      <c r="L3" t="n">
         <v>2019</v>
       </c>
-      <c r="H3" s="2" t="n">
+      <c r="M3" s="4" t="n">
         <v>45397</v>
       </c>
-      <c r="I3" t="n">
+      <c r="N3" t="n">
         <v>50</v>
       </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="n">
+      <c r="O3" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="P3" t="n">
         <v>80</v>
       </c>
-      <c r="L3" t="n">
+      <c r="Q3" t="n">
         <v>18</v>
       </c>
-      <c r="M3" t="n">
+      <c r="R3" t="n">
         <v>225</v>
       </c>
-      <c r="N3" t="n">
+      <c r="S3" t="n">
         <v>60</v>
       </c>
-      <c r="O3" t="n">
+      <c r="T3" t="n">
         <v>160</v>
       </c>
-      <c r="P3" t="n">
+      <c r="U3" t="n">
         <v>45</v>
       </c>
-      <c r="Q3" t="n">
+      <c r="V3" t="n">
         <v>540</v>
       </c>
-      <c r="R3" t="n">
+      <c r="W3" t="n">
         <v>70</v>
       </c>
-      <c r="S3" t="n">
+      <c r="X3" t="n">
+        <v>130</v>
+      </c>
+      <c r="Y3" t="n">
         <v>0</v>
       </c>
-      <c r="T3" t="n">
-        <v>0</v>
-      </c>
-      <c r="U3" t="n">
+      <c r="Z3" t="n">
         <v>0.24</v>
+      </c>
+      <c r="AA3" t="n">
+        <v>620</v>
+      </c>
+      <c r="AB3" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="AC3" t="n">
+        <v>2</v>
+      </c>
+      <c r="AD3" t="n">
+        <v>1.4</v>
       </c>
     </row>
     <row r="4">
@@ -703,7 +832,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Western Europe</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -711,51 +840,90 @@
           <t>Fully Realized</t>
         </is>
       </c>
-      <c r="F4" s="2" t="n">
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Strategic Sale</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>R. Patel</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Common Equity</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Carve-out</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Broad Auction</t>
+        </is>
+      </c>
+      <c r="K4" s="4" t="n">
         <v>42887</v>
       </c>
-      <c r="G4" t="n">
+      <c r="L4" t="n">
         <v>2017</v>
       </c>
-      <c r="H4" s="2" t="n">
+      <c r="M4" s="4" t="n">
         <v>44834</v>
       </c>
-      <c r="I4" t="n">
+      <c r="N4" t="n">
         <v>60</v>
       </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="n">
+      <c r="O4" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="P4" t="n">
         <v>200</v>
       </c>
-      <c r="L4" t="n">
+      <c r="Q4" t="n">
         <v>35</v>
       </c>
-      <c r="M4" t="n">
+      <c r="R4" t="n">
         <v>380</v>
       </c>
-      <c r="N4" t="n">
+      <c r="S4" t="n">
         <v>120</v>
       </c>
-      <c r="O4" t="n">
+      <c r="T4" t="n">
         <v>310</v>
       </c>
-      <c r="P4" t="n">
+      <c r="U4" t="n">
         <v>58</v>
       </c>
-      <c r="Q4" t="n">
+      <c r="V4" t="n">
         <v>620</v>
       </c>
-      <c r="R4" t="n">
+      <c r="W4" t="n">
         <v>110</v>
       </c>
-      <c r="S4" t="n">
+      <c r="X4" t="n">
+        <v>118</v>
+      </c>
+      <c r="Y4" t="n">
         <v>0</v>
       </c>
-      <c r="T4" t="n">
-        <v>0</v>
-      </c>
-      <c r="U4" t="n">
+      <c r="Z4" t="n">
         <v>0.2</v>
+      </c>
+      <c r="AA4" t="n">
+        <v>550</v>
+      </c>
+      <c r="AB4" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="AC4" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="AD4" t="n">
+        <v>1.2</v>
       </c>
     </row>
     <row r="5">
@@ -776,7 +944,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>US</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -784,51 +952,90 @@
           <t>Fully Realized</t>
         </is>
       </c>
-      <c r="F5" s="2" t="n">
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Secondary Buyout</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>M. Rivera</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>Common Equity</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Platform</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Proprietary</t>
+        </is>
+      </c>
+      <c r="K5" s="4" t="n">
         <v>42694</v>
       </c>
-      <c r="G5" t="n">
+      <c r="L5" t="n">
         <v>2016</v>
       </c>
-      <c r="H5" s="2" t="n">
+      <c r="M5" s="4" t="n">
         <v>44270</v>
       </c>
-      <c r="I5" t="n">
+      <c r="N5" t="n">
         <v>40</v>
       </c>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="n">
+      <c r="O5" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="P5" t="n">
         <v>65</v>
       </c>
-      <c r="L5" t="n">
+      <c r="Q5" t="n">
         <v>12</v>
       </c>
-      <c r="M5" t="n">
+      <c r="R5" t="n">
         <v>140</v>
       </c>
-      <c r="N5" t="n">
+      <c r="S5" t="n">
         <v>35</v>
       </c>
-      <c r="O5" t="n">
+      <c r="T5" t="n">
         <v>95</v>
       </c>
-      <c r="P5" t="n">
+      <c r="U5" t="n">
         <v>22</v>
       </c>
-      <c r="Q5" t="n">
+      <c r="V5" t="n">
         <v>260</v>
       </c>
-      <c r="R5" t="n">
+      <c r="W5" t="n">
         <v>30</v>
       </c>
-      <c r="S5" t="n">
+      <c r="X5" t="n">
+        <v>72</v>
+      </c>
+      <c r="Y5" t="n">
         <v>0</v>
       </c>
-      <c r="T5" t="n">
-        <v>0</v>
-      </c>
-      <c r="U5" t="n">
+      <c r="Z5" t="n">
         <v>0.18</v>
+      </c>
+      <c r="AA5" t="n">
+        <v>550</v>
+      </c>
+      <c r="AB5" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="AC5" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="AD5" t="n">
+        <v>1.2</v>
       </c>
     </row>
     <row r="6">
@@ -849,7 +1056,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>US</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -857,51 +1064,90 @@
           <t>Fully Realized</t>
         </is>
       </c>
-      <c r="F6" s="2" t="n">
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>Recapitalization</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>T. Brooks</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>Convertible Preferred</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Turnaround</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Broad Auction</t>
+        </is>
+      </c>
+      <c r="K6" s="4" t="n">
         <v>42826</v>
       </c>
-      <c r="G6" t="n">
+      <c r="L6" t="n">
         <v>2017</v>
       </c>
-      <c r="H6" s="2" t="n">
+      <c r="M6" s="4" t="n">
         <v>44926</v>
       </c>
-      <c r="I6" t="n">
+      <c r="N6" t="n">
         <v>55</v>
       </c>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="n">
+      <c r="O6" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="P6" t="n">
         <v>150</v>
       </c>
-      <c r="L6" t="n">
+      <c r="Q6" t="n">
         <v>25</v>
       </c>
-      <c r="M6" t="n">
+      <c r="R6" t="n">
         <v>280</v>
       </c>
-      <c r="N6" t="n">
+      <c r="S6" t="n">
         <v>75</v>
       </c>
-      <c r="O6" t="n">
+      <c r="T6" t="n">
         <v>130</v>
       </c>
-      <c r="P6" t="n">
+      <c r="U6" t="n">
         <v>20</v>
       </c>
-      <c r="Q6" t="n">
+      <c r="V6" t="n">
         <v>230</v>
       </c>
-      <c r="R6" t="n">
+      <c r="W6" t="n">
         <v>80</v>
       </c>
-      <c r="S6" t="n">
+      <c r="X6" t="n">
+        <v>45</v>
+      </c>
+      <c r="Y6" t="n">
         <v>0</v>
       </c>
-      <c r="T6" t="n">
-        <v>0</v>
-      </c>
-      <c r="U6" t="n">
+      <c r="Z6" t="n">
         <v>-0.03</v>
+      </c>
+      <c r="AA6" t="n">
+        <v>550</v>
+      </c>
+      <c r="AB6" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="AC6" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="AD6" t="n">
+        <v>1.2</v>
       </c>
     </row>
     <row r="7">
@@ -922,7 +1168,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>US</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -930,51 +1176,90 @@
           <t>Partially Realized</t>
         </is>
       </c>
-      <c r="F7" s="2" t="n">
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>Minority Recap</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>L. Chen</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>Common Equity</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Platform</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Proprietary</t>
+        </is>
+      </c>
+      <c r="K7" s="4" t="n">
         <v>44027</v>
       </c>
-      <c r="G7" t="n">
+      <c r="L7" t="n">
         <v>2020</v>
       </c>
-      <c r="H7" s="2" t="n">
+      <c r="M7" s="4" t="n">
         <v>45505</v>
       </c>
-      <c r="I7" t="n">
+      <c r="N7" t="n">
         <v>85</v>
       </c>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="n">
+      <c r="O7" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="P7" t="n">
         <v>45</v>
       </c>
-      <c r="L7" t="n">
+      <c r="Q7" t="n">
         <v>8</v>
       </c>
-      <c r="M7" t="n">
+      <c r="R7" t="n">
         <v>190</v>
       </c>
-      <c r="N7" t="n">
+      <c r="S7" t="n">
         <v>40</v>
       </c>
-      <c r="O7" t="n">
+      <c r="T7" t="n">
         <v>130</v>
       </c>
-      <c r="P7" t="n">
+      <c r="U7" t="n">
         <v>35</v>
       </c>
-      <c r="Q7" t="n">
+      <c r="V7" t="n">
         <v>520</v>
       </c>
-      <c r="R7" t="n">
+      <c r="W7" t="n">
         <v>55</v>
       </c>
-      <c r="S7" t="n">
-        <v>0</v>
-      </c>
-      <c r="T7" t="n">
-        <v>0</v>
-      </c>
-      <c r="U7" t="n">
+      <c r="X7" t="n">
+        <v>90</v>
+      </c>
+      <c r="Y7" t="n">
+        <v>75</v>
+      </c>
+      <c r="Z7" t="n">
         <v>0.3</v>
+      </c>
+      <c r="AA7" t="n">
+        <v>710</v>
+      </c>
+      <c r="AB7" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="AC7" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="AD7" t="n">
+        <v>1.6</v>
       </c>
     </row>
     <row r="8">
@@ -995,7 +1280,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Western Europe</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -1003,49 +1288,87 @@
           <t>Partially Realized</t>
         </is>
       </c>
-      <c r="F8" s="2" t="n">
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>IPO (Partial Exit)</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>A. Morgan</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Preferred Equity</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Growth Buyout</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Limited Auction</t>
+        </is>
+      </c>
+      <c r="K8" s="4" t="n">
         <v>43709</v>
       </c>
-      <c r="G8" t="n">
+      <c r="L8" t="n">
         <v>2019</v>
       </c>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="n">
+      <c r="N8" t="n">
         <v>65</v>
       </c>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="n">
+      <c r="O8" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="P8" t="n">
         <v>55</v>
       </c>
-      <c r="L8" t="n">
+      <c r="Q8" t="n">
         <v>10</v>
       </c>
-      <c r="M8" t="n">
+      <c r="R8" t="n">
         <v>160</v>
       </c>
-      <c r="N8" t="n">
+      <c r="S8" t="n">
         <v>45</v>
       </c>
-      <c r="O8" t="n">
+      <c r="T8" t="n">
         <v>110</v>
       </c>
-      <c r="P8" t="n">
+      <c r="U8" t="n">
         <v>28</v>
       </c>
-      <c r="Q8" t="n">
+      <c r="V8" t="n">
         <v>390</v>
       </c>
-      <c r="R8" t="n">
+      <c r="W8" t="n">
         <v>50</v>
       </c>
-      <c r="S8" t="n">
-        <v>0</v>
-      </c>
-      <c r="T8" t="n">
-        <v>0</v>
-      </c>
-      <c r="U8" t="n">
+      <c r="X8" t="n">
+        <v>40</v>
+      </c>
+      <c r="Y8" t="n">
+        <v>82</v>
+      </c>
+      <c r="Z8" t="n">
         <v>0.16</v>
+      </c>
+      <c r="AA8" t="n">
+        <v>620</v>
+      </c>
+      <c r="AB8" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="AC8" t="n">
+        <v>2</v>
+      </c>
+      <c r="AD8" t="n">
+        <v>1.4</v>
       </c>
     </row>
     <row r="9">
@@ -1066,7 +1389,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>US</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -1074,49 +1397,87 @@
           <t>Unrealized</t>
         </is>
       </c>
-      <c r="F9" s="2" t="n">
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>Unrealized / N.A.</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>S. Nguyen</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Preferred Equity</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Platform</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Proprietary</t>
+        </is>
+      </c>
+      <c r="K9" s="4" t="n">
         <v>44256</v>
       </c>
-      <c r="G9" t="n">
+      <c r="L9" t="n">
         <v>2021</v>
       </c>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="n">
+      <c r="N9" t="n">
         <v>100</v>
       </c>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="n">
+      <c r="O9" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="P9" t="n">
         <v>30</v>
       </c>
-      <c r="L9" t="n">
+      <c r="Q9" t="n">
         <v>5</v>
       </c>
-      <c r="M9" t="n">
+      <c r="R9" t="n">
         <v>150</v>
       </c>
-      <c r="N9" t="n">
+      <c r="S9" t="n">
         <v>20</v>
       </c>
-      <c r="O9" t="n">
+      <c r="T9" t="n">
         <v>85</v>
       </c>
-      <c r="P9" t="n">
+      <c r="U9" t="n">
         <v>22</v>
       </c>
-      <c r="Q9" t="n">
+      <c r="V9" t="n">
         <v>400</v>
       </c>
-      <c r="R9" t="n">
+      <c r="W9" t="n">
         <v>35</v>
       </c>
-      <c r="S9" t="n">
+      <c r="X9" t="n">
         <v>0</v>
       </c>
-      <c r="T9" t="n">
-        <v>0</v>
-      </c>
-      <c r="U9" t="n">
+      <c r="Y9" t="n">
+        <v>195</v>
+      </c>
+      <c r="Z9" t="n">
         <v>0.15</v>
+      </c>
+      <c r="AA9" t="n">
+        <v>710</v>
+      </c>
+      <c r="AB9" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="AC9" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="AD9" t="n">
+        <v>1.6</v>
       </c>
     </row>
     <row r="10">
@@ -1137,7 +1498,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -1145,49 +1506,87 @@
           <t>Unrealized</t>
         </is>
       </c>
-      <c r="F10" s="2" t="n">
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>Unrealized / N.A.</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>R. Patel</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Structured Equity</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Platform</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Bilateral</t>
+        </is>
+      </c>
+      <c r="K10" s="4" t="n">
         <v>44576</v>
       </c>
-      <c r="G10" t="n">
+      <c r="L10" t="n">
         <v>2022</v>
       </c>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="n">
+      <c r="N10" t="n">
         <v>70</v>
       </c>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="n">
+      <c r="O10" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="P10" t="n">
         <v>90</v>
       </c>
-      <c r="L10" t="n">
+      <c r="Q10" t="n">
         <v>18</v>
       </c>
-      <c r="M10" t="n">
+      <c r="R10" t="n">
         <v>210</v>
       </c>
-      <c r="N10" t="n">
+      <c r="S10" t="n">
         <v>55</v>
       </c>
-      <c r="O10" t="n">
+      <c r="T10" t="n">
         <v>140</v>
       </c>
-      <c r="P10" t="n">
+      <c r="U10" t="n">
         <v>30</v>
       </c>
-      <c r="Q10" t="n">
+      <c r="V10" t="n">
         <v>350</v>
       </c>
-      <c r="R10" t="n">
+      <c r="W10" t="n">
         <v>60</v>
       </c>
-      <c r="S10" t="n">
+      <c r="X10" t="n">
         <v>0</v>
       </c>
-      <c r="T10" t="n">
-        <v>0</v>
-      </c>
-      <c r="U10" t="n">
+      <c r="Y10" t="n">
+        <v>84</v>
+      </c>
+      <c r="Z10" t="n">
         <v>0.12</v>
+      </c>
+      <c r="AA10" t="n">
+        <v>710</v>
+      </c>
+      <c r="AB10" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="AC10" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="AD10" t="n">
+        <v>1.6</v>
       </c>
     </row>
     <row r="11">
@@ -1208,7 +1607,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>APAC</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1216,49 +1615,87 @@
           <t>Unrealized</t>
         </is>
       </c>
-      <c r="F11" s="2" t="n">
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>Unrealized / N.A.</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>M. Rivera</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Common Equity</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Platform</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Broad Auction</t>
+        </is>
+      </c>
+      <c r="K11" s="4" t="n">
         <v>45078</v>
       </c>
-      <c r="G11" t="n">
+      <c r="L11" t="n">
         <v>2023</v>
-      </c>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="n">
-        <v>90</v>
-      </c>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="n">
-        <v>180</v>
-      </c>
-      <c r="L11" t="n">
-        <v>32</v>
-      </c>
-      <c r="M11" t="n">
-        <v>350</v>
       </c>
       <c r="N11" t="n">
         <v>90</v>
       </c>
       <c r="O11" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="P11" t="n">
+        <v>180</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>32</v>
+      </c>
+      <c r="R11" t="n">
+        <v>350</v>
+      </c>
+      <c r="S11" t="n">
+        <v>90</v>
+      </c>
+      <c r="T11" t="n">
         <v>210</v>
       </c>
-      <c r="P11" t="n">
+      <c r="U11" t="n">
         <v>38</v>
       </c>
-      <c r="Q11" t="n">
+      <c r="V11" t="n">
         <v>420</v>
       </c>
-      <c r="R11" t="n">
+      <c r="W11" t="n">
         <v>85</v>
       </c>
-      <c r="S11" t="n">
+      <c r="X11" t="n">
         <v>0</v>
       </c>
-      <c r="T11" t="n">
-        <v>0</v>
-      </c>
-      <c r="U11" t="n">
+      <c r="Y11" t="n">
+        <v>162</v>
+      </c>
+      <c r="Z11" t="n">
         <v>0.1</v>
+      </c>
+      <c r="AA11" t="n">
+        <v>805</v>
+      </c>
+      <c r="AB11" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="AC11" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="AD11" t="n">
+        <v>1.8</v>
       </c>
     </row>
     <row r="12">
@@ -1279,7 +1716,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>US</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1287,49 +1724,87 @@
           <t>Unrealized</t>
         </is>
       </c>
-      <c r="F12" s="2" t="n">
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>Unrealized / N.A.</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>T. Brooks</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Common Equity</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Platform</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Limited Auction</t>
+        </is>
+      </c>
+      <c r="K12" s="4" t="n">
         <v>45184</v>
       </c>
-      <c r="G12" t="n">
+      <c r="L12" t="n">
         <v>2023</v>
       </c>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="n">
+      <c r="N12" t="n">
         <v>80</v>
       </c>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="n">
+      <c r="O12" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="P12" t="n">
         <v>60</v>
       </c>
-      <c r="L12" t="n">
+      <c r="Q12" t="n">
         <v>15</v>
       </c>
-      <c r="M12" t="n">
+      <c r="R12" t="n">
         <v>175</v>
       </c>
-      <c r="N12" t="n">
+      <c r="S12" t="n">
         <v>30</v>
       </c>
-      <c r="O12" t="n">
+      <c r="T12" t="n">
         <v>72</v>
       </c>
-      <c r="P12" t="n">
+      <c r="U12" t="n">
         <v>19</v>
       </c>
-      <c r="Q12" t="n">
+      <c r="V12" t="n">
         <v>220</v>
       </c>
-      <c r="R12" t="n">
+      <c r="W12" t="n">
         <v>28</v>
       </c>
-      <c r="S12" t="n">
+      <c r="X12" t="n">
         <v>0</v>
       </c>
-      <c r="T12" t="n">
-        <v>0</v>
-      </c>
-      <c r="U12" t="n">
+      <c r="Y12" t="n">
+        <v>104</v>
+      </c>
+      <c r="Z12" t="n">
         <v>0.08</v>
+      </c>
+      <c r="AA12" t="n">
+        <v>805</v>
+      </c>
+      <c r="AB12" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="AC12" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="AD12" t="n">
+        <v>1.8</v>
       </c>
     </row>
     <row r="13">
@@ -1350,7 +1825,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1358,48 +1833,443 @@
           <t>Unrealized</t>
         </is>
       </c>
-      <c r="F13" s="2" t="n">
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>Unrealized / N.A.</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>S. Nguyen</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Preferred Equity</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Growth Buyout</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Proprietary</t>
+        </is>
+      </c>
+      <c r="K13" s="4" t="n">
         <v>45323</v>
       </c>
-      <c r="G13" t="n">
+      <c r="L13" t="n">
         <v>2024</v>
       </c>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="n">
+      <c r="N13" t="n">
         <v>110</v>
       </c>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="n">
+      <c r="O13" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="P13" t="n">
         <v>25</v>
       </c>
-      <c r="L13" t="n">
+      <c r="Q13" t="n">
         <v>3</v>
       </c>
-      <c r="M13" t="n">
+      <c r="R13" t="n">
         <v>120</v>
       </c>
-      <c r="N13" t="n">
+      <c r="S13" t="n">
         <v>15</v>
       </c>
-      <c r="O13" t="n">
+      <c r="T13" t="n">
         <v>35</v>
       </c>
-      <c r="P13" t="n">
+      <c r="U13" t="n">
         <v>6</v>
       </c>
-      <c r="Q13" t="n">
+      <c r="V13" t="n">
         <v>180</v>
       </c>
-      <c r="R13" t="n">
+      <c r="W13" t="n">
         <v>18</v>
       </c>
-      <c r="S13" t="n">
+      <c r="X13" t="n">
         <v>0</v>
       </c>
-      <c r="T13" t="n">
+      <c r="Y13" t="n">
+        <v>176</v>
+      </c>
+      <c r="AA13" t="n">
+        <v>805</v>
+      </c>
+      <c r="AB13" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="AC13" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="AD13" t="n">
+        <v>1.8</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Company Name</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Fund</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Event Date</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Event Type</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Cardinal Commerce</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Fund VII</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>2013-03-31</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Capital Call</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>-5</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Initial draw</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Company Name</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Fund</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Quarter End</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>EBITDA</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Enterprise Value</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Net Debt</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Equity Value</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Valuation Basis</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Cardinal Commerce</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Fund VII</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>2014-12-31</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>72</v>
+      </c>
+      <c r="E2" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="F2" t="n">
+        <v>155</v>
+      </c>
+      <c r="G2" t="n">
+        <v>40</v>
+      </c>
+      <c r="H2" t="n">
+        <v>115</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Quarterly Mark</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Finance Team</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Fund</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Quarter End</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Committed Capital</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Paid In Capital</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Distributed Capital</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>NAV</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Unfunded Commitment</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Fund VII</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2016-12-31</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>353</v>
+      </c>
+      <c r="D2" t="n">
+        <v>278.3</v>
+      </c>
+      <c r="E2" t="n">
+        <v>1078.9</v>
+      </c>
+      <c r="F2" t="n">
         <v>0</v>
       </c>
-      <c r="U13" t="inlineStr"/>
+      <c r="G2" t="n">
+        <v>74.7</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Company Name</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Fund</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Baseline Date</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Target IRR</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Target MOIC</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Target Hold Years</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Target Exit Multiple</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Target Revenue CAGR</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Target EBITDA CAGR</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Cardinal Commerce</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Fund VII</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>2012-12-01</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E2" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="F2" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="G2" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0.1</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add first-class firm scope with global firm switching
</commit_message>
<xml_diff>
--- a/PE_Fund_Data_Template.xlsx
+++ b/PE_Fund_Data_Template.xlsx
@@ -435,156 +435,161 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD13"/>
+  <dimension ref="A1:AE13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>Firm Name</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
           <t>Company Name</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Fund</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Sector</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Geography</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Exit Type</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Lead Partner</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Security Type</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Deal Type</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Entry Channel</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Investment Date</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Year Invested</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Exit Date</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Equity Invested</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Ownership %</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Entry Revenue</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Entry EBITDA</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Entry EV</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Entry Net Debt</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Exit Revenue</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Exit EBITDA</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>Exit EV</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>Exit Net Debt</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>Realized Value</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>Unrealized Value</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>IRR</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>Fund Size</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>Net IRR</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>Net MOIC</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>DPI</t>
         </is>
@@ -593,1323 +598,1383 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>Example Firm</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
           <t>Apex Healthcare Solutions</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>Fund III</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>Healthcare</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>US</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>Fully Realized</t>
         </is>
       </c>
-      <c r="F2" s="3" t="inlineStr">
+      <c r="G2" s="3" t="inlineStr">
         <is>
           <t>Strategic Sale</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>A. Morgan</t>
         </is>
       </c>
-      <c r="H2" s="3" t="inlineStr">
+      <c r="I2" s="3" t="inlineStr">
         <is>
           <t>Common Equity</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>Platform</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>Proprietary</t>
         </is>
       </c>
-      <c r="K2" s="4" t="n">
+      <c r="L2" s="4" t="n">
         <v>43174</v>
       </c>
-      <c r="L2" t="n">
+      <c r="M2" t="n">
         <v>2018</v>
       </c>
-      <c r="M2" s="4" t="n">
+      <c r="N2" s="4" t="n">
         <v>45107</v>
       </c>
-      <c r="N2" t="n">
+      <c r="O2" t="n">
         <v>75</v>
       </c>
-      <c r="O2" t="n">
+      <c r="P2" t="n">
         <v>0.42</v>
       </c>
-      <c r="P2" t="n">
+      <c r="Q2" t="n">
         <v>120</v>
       </c>
-      <c r="Q2" t="n">
+      <c r="R2" t="n">
         <v>28</v>
       </c>
-      <c r="R2" t="n">
+      <c r="S2" t="n">
         <v>310</v>
       </c>
-      <c r="S2" t="n">
+      <c r="T2" t="n">
         <v>85</v>
       </c>
-      <c r="T2" t="n">
+      <c r="U2" t="n">
         <v>245</v>
       </c>
-      <c r="U2" t="n">
+      <c r="V2" t="n">
         <v>62</v>
       </c>
-      <c r="V2" t="n">
+      <c r="W2" t="n">
         <v>720</v>
       </c>
-      <c r="W2" t="n">
+      <c r="X2" t="n">
         <v>95</v>
       </c>
-      <c r="X2" t="n">
+      <c r="Y2" t="n">
         <v>170</v>
       </c>
-      <c r="Y2" t="n">
+      <c r="Z2" t="n">
         <v>0</v>
       </c>
-      <c r="Z2" t="n">
+      <c r="AA2" t="n">
         <v>0.28</v>
       </c>
-      <c r="AA2" t="n">
+      <c r="AB2" t="n">
         <v>620</v>
       </c>
-      <c r="AB2" t="n">
+      <c r="AC2" t="n">
         <v>0.2</v>
       </c>
-      <c r="AC2" t="n">
+      <c r="AD2" t="n">
         <v>2</v>
       </c>
-      <c r="AD2" t="n">
+      <c r="AE2" t="n">
         <v>1.4</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>Example Firm</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
           <t>TechVault Software</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>Fund III</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>Technology</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>US</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>Fully Realized</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t>Secondary Buyout</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>L. Chen</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr">
+      <c r="I3" s="3" t="inlineStr">
         <is>
           <t>Preferred Equity</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>Platform</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>Limited Auction</t>
         </is>
       </c>
-      <c r="K3" s="4" t="n">
+      <c r="L3" s="4" t="n">
         <v>43475</v>
       </c>
-      <c r="L3" t="n">
+      <c r="M3" t="n">
         <v>2019</v>
       </c>
-      <c r="M3" s="4" t="n">
+      <c r="N3" s="4" t="n">
         <v>45397</v>
       </c>
-      <c r="N3" t="n">
+      <c r="O3" t="n">
         <v>50</v>
       </c>
-      <c r="O3" t="n">
+      <c r="P3" t="n">
         <v>0.35</v>
       </c>
-      <c r="P3" t="n">
+      <c r="Q3" t="n">
         <v>80</v>
       </c>
-      <c r="Q3" t="n">
+      <c r="R3" t="n">
         <v>18</v>
       </c>
-      <c r="R3" t="n">
+      <c r="S3" t="n">
         <v>225</v>
       </c>
-      <c r="S3" t="n">
+      <c r="T3" t="n">
         <v>60</v>
       </c>
-      <c r="T3" t="n">
+      <c r="U3" t="n">
         <v>160</v>
       </c>
-      <c r="U3" t="n">
+      <c r="V3" t="n">
         <v>45</v>
       </c>
-      <c r="V3" t="n">
+      <c r="W3" t="n">
         <v>540</v>
       </c>
-      <c r="W3" t="n">
+      <c r="X3" t="n">
         <v>70</v>
       </c>
-      <c r="X3" t="n">
+      <c r="Y3" t="n">
         <v>130</v>
       </c>
-      <c r="Y3" t="n">
+      <c r="Z3" t="n">
         <v>0</v>
       </c>
-      <c r="Z3" t="n">
+      <c r="AA3" t="n">
         <v>0.24</v>
       </c>
-      <c r="AA3" t="n">
+      <c r="AB3" t="n">
         <v>620</v>
       </c>
-      <c r="AB3" t="n">
+      <c r="AC3" t="n">
         <v>0.2</v>
       </c>
-      <c r="AC3" t="n">
+      <c r="AD3" t="n">
         <v>2</v>
       </c>
-      <c r="AD3" t="n">
+      <c r="AE3" t="n">
         <v>1.4</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>Example Firm</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
           <t>National Logistics Group</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>Fund II</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>Industrials</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>Western Europe</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>Fully Realized</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>Strategic Sale</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>R. Patel</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="I4" s="3" t="inlineStr">
         <is>
           <t>Common Equity</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>Carve-out</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>Broad Auction</t>
         </is>
       </c>
-      <c r="K4" s="4" t="n">
+      <c r="L4" s="4" t="n">
         <v>42887</v>
       </c>
-      <c r="L4" t="n">
+      <c r="M4" t="n">
         <v>2017</v>
       </c>
-      <c r="M4" s="4" t="n">
+      <c r="N4" s="4" t="n">
         <v>44834</v>
       </c>
-      <c r="N4" t="n">
+      <c r="O4" t="n">
         <v>60</v>
       </c>
-      <c r="O4" t="n">
+      <c r="P4" t="n">
         <v>0.28</v>
       </c>
-      <c r="P4" t="n">
+      <c r="Q4" t="n">
         <v>200</v>
       </c>
-      <c r="Q4" t="n">
+      <c r="R4" t="n">
         <v>35</v>
       </c>
-      <c r="R4" t="n">
+      <c r="S4" t="n">
         <v>380</v>
       </c>
-      <c r="S4" t="n">
+      <c r="T4" t="n">
         <v>120</v>
       </c>
-      <c r="T4" t="n">
+      <c r="U4" t="n">
         <v>310</v>
       </c>
-      <c r="U4" t="n">
+      <c r="V4" t="n">
         <v>58</v>
       </c>
-      <c r="V4" t="n">
+      <c r="W4" t="n">
         <v>620</v>
       </c>
-      <c r="W4" t="n">
+      <c r="X4" t="n">
         <v>110</v>
       </c>
-      <c r="X4" t="n">
+      <c r="Y4" t="n">
         <v>118</v>
       </c>
-      <c r="Y4" t="n">
+      <c r="Z4" t="n">
         <v>0</v>
       </c>
-      <c r="Z4" t="n">
+      <c r="AA4" t="n">
         <v>0.2</v>
       </c>
-      <c r="AA4" t="n">
+      <c r="AB4" t="n">
         <v>550</v>
       </c>
-      <c r="AB4" t="n">
+      <c r="AC4" t="n">
         <v>0.18</v>
       </c>
-      <c r="AC4" t="n">
+      <c r="AD4" t="n">
         <v>1.8</v>
       </c>
-      <c r="AD4" t="n">
+      <c r="AE4" t="n">
         <v>1.2</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>Example Firm</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
           <t>Summit Education Partners</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>Fund II</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>Consumer</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>US</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>Fully Realized</t>
         </is>
       </c>
-      <c r="F5" s="3" t="inlineStr">
+      <c r="G5" s="3" t="inlineStr">
         <is>
           <t>Secondary Buyout</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>M. Rivera</t>
         </is>
       </c>
-      <c r="H5" s="3" t="inlineStr">
+      <c r="I5" s="3" t="inlineStr">
         <is>
           <t>Common Equity</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="J5" t="inlineStr">
         <is>
           <t>Platform</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>Proprietary</t>
         </is>
       </c>
-      <c r="K5" s="4" t="n">
+      <c r="L5" s="4" t="n">
         <v>42694</v>
       </c>
-      <c r="L5" t="n">
+      <c r="M5" t="n">
         <v>2016</v>
       </c>
-      <c r="M5" s="4" t="n">
+      <c r="N5" s="4" t="n">
         <v>44270</v>
       </c>
-      <c r="N5" t="n">
+      <c r="O5" t="n">
         <v>40</v>
       </c>
-      <c r="O5" t="n">
+      <c r="P5" t="n">
         <v>0.31</v>
       </c>
-      <c r="P5" t="n">
+      <c r="Q5" t="n">
         <v>65</v>
       </c>
-      <c r="Q5" t="n">
+      <c r="R5" t="n">
         <v>12</v>
       </c>
-      <c r="R5" t="n">
+      <c r="S5" t="n">
         <v>140</v>
       </c>
-      <c r="S5" t="n">
+      <c r="T5" t="n">
         <v>35</v>
       </c>
-      <c r="T5" t="n">
+      <c r="U5" t="n">
         <v>95</v>
       </c>
-      <c r="U5" t="n">
+      <c r="V5" t="n">
         <v>22</v>
       </c>
-      <c r="V5" t="n">
+      <c r="W5" t="n">
         <v>260</v>
       </c>
-      <c r="W5" t="n">
+      <c r="X5" t="n">
         <v>30</v>
       </c>
-      <c r="X5" t="n">
+      <c r="Y5" t="n">
         <v>72</v>
       </c>
-      <c r="Y5" t="n">
+      <c r="Z5" t="n">
         <v>0</v>
       </c>
-      <c r="Z5" t="n">
+      <c r="AA5" t="n">
         <v>0.18</v>
       </c>
-      <c r="AA5" t="n">
+      <c r="AB5" t="n">
         <v>550</v>
       </c>
-      <c r="AB5" t="n">
+      <c r="AC5" t="n">
         <v>0.18</v>
       </c>
-      <c r="AC5" t="n">
+      <c r="AD5" t="n">
         <v>1.8</v>
       </c>
-      <c r="AD5" t="n">
+      <c r="AE5" t="n">
         <v>1.2</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>Example Firm</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
           <t>BrightPath Retail</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>Fund II</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>Consumer</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>US</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>Fully Realized</t>
         </is>
       </c>
-      <c r="F6" s="3" t="inlineStr">
+      <c r="G6" s="3" t="inlineStr">
         <is>
           <t>Recapitalization</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>T. Brooks</t>
         </is>
       </c>
-      <c r="H6" s="3" t="inlineStr">
+      <c r="I6" s="3" t="inlineStr">
         <is>
           <t>Convertible Preferred</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="J6" t="inlineStr">
         <is>
           <t>Turnaround</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="K6" t="inlineStr">
         <is>
           <t>Broad Auction</t>
         </is>
       </c>
-      <c r="K6" s="4" t="n">
+      <c r="L6" s="4" t="n">
         <v>42826</v>
       </c>
-      <c r="L6" t="n">
+      <c r="M6" t="n">
         <v>2017</v>
       </c>
-      <c r="M6" s="4" t="n">
+      <c r="N6" s="4" t="n">
         <v>44926</v>
       </c>
-      <c r="N6" t="n">
+      <c r="O6" t="n">
         <v>55</v>
       </c>
-      <c r="O6" t="n">
+      <c r="P6" t="n">
         <v>0.4</v>
       </c>
-      <c r="P6" t="n">
+      <c r="Q6" t="n">
         <v>150</v>
       </c>
-      <c r="Q6" t="n">
+      <c r="R6" t="n">
         <v>25</v>
       </c>
-      <c r="R6" t="n">
+      <c r="S6" t="n">
         <v>280</v>
       </c>
-      <c r="S6" t="n">
+      <c r="T6" t="n">
         <v>75</v>
       </c>
-      <c r="T6" t="n">
+      <c r="U6" t="n">
         <v>130</v>
       </c>
-      <c r="U6" t="n">
+      <c r="V6" t="n">
         <v>20</v>
       </c>
-      <c r="V6" t="n">
+      <c r="W6" t="n">
         <v>230</v>
       </c>
-      <c r="W6" t="n">
+      <c r="X6" t="n">
         <v>80</v>
       </c>
-      <c r="X6" t="n">
+      <c r="Y6" t="n">
         <v>45</v>
       </c>
-      <c r="Y6" t="n">
+      <c r="Z6" t="n">
         <v>0</v>
       </c>
-      <c r="Z6" t="n">
+      <c r="AA6" t="n">
         <v>-0.03</v>
       </c>
-      <c r="AA6" t="n">
+      <c r="AB6" t="n">
         <v>550</v>
       </c>
-      <c r="AB6" t="n">
+      <c r="AC6" t="n">
         <v>0.18</v>
       </c>
-      <c r="AC6" t="n">
+      <c r="AD6" t="n">
         <v>1.8</v>
       </c>
-      <c r="AD6" t="n">
+      <c r="AE6" t="n">
         <v>1.2</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>Example Firm</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
           <t>CloudBridge Analytics</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>Fund IV</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>Technology</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>US</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>Partially Realized</t>
         </is>
       </c>
-      <c r="F7" s="3" t="inlineStr">
+      <c r="G7" s="3" t="inlineStr">
         <is>
           <t>Minority Recap</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="H7" t="inlineStr">
         <is>
           <t>L. Chen</t>
         </is>
       </c>
-      <c r="H7" s="3" t="inlineStr">
+      <c r="I7" s="3" t="inlineStr">
         <is>
           <t>Common Equity</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="J7" t="inlineStr">
         <is>
           <t>Platform</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="K7" t="inlineStr">
         <is>
           <t>Proprietary</t>
         </is>
       </c>
-      <c r="K7" s="4" t="n">
+      <c r="L7" s="4" t="n">
         <v>44027</v>
       </c>
-      <c r="L7" t="n">
+      <c r="M7" t="n">
         <v>2020</v>
       </c>
-      <c r="M7" s="4" t="n">
+      <c r="N7" s="4" t="n">
         <v>45505</v>
       </c>
-      <c r="N7" t="n">
+      <c r="O7" t="n">
         <v>85</v>
       </c>
-      <c r="O7" t="n">
+      <c r="P7" t="n">
         <v>0.33</v>
       </c>
-      <c r="P7" t="n">
+      <c r="Q7" t="n">
         <v>45</v>
       </c>
-      <c r="Q7" t="n">
+      <c r="R7" t="n">
         <v>8</v>
       </c>
-      <c r="R7" t="n">
+      <c r="S7" t="n">
         <v>190</v>
       </c>
-      <c r="S7" t="n">
+      <c r="T7" t="n">
         <v>40</v>
       </c>
-      <c r="T7" t="n">
+      <c r="U7" t="n">
         <v>130</v>
       </c>
-      <c r="U7" t="n">
+      <c r="V7" t="n">
         <v>35</v>
       </c>
-      <c r="V7" t="n">
+      <c r="W7" t="n">
         <v>520</v>
       </c>
-      <c r="W7" t="n">
+      <c r="X7" t="n">
         <v>55</v>
       </c>
-      <c r="X7" t="n">
+      <c r="Y7" t="n">
         <v>90</v>
       </c>
-      <c r="Y7" t="n">
+      <c r="Z7" t="n">
         <v>75</v>
       </c>
-      <c r="Z7" t="n">
+      <c r="AA7" t="n">
         <v>0.3</v>
       </c>
-      <c r="AA7" t="n">
+      <c r="AB7" t="n">
         <v>710</v>
       </c>
-      <c r="AB7" t="n">
+      <c r="AC7" t="n">
         <v>0.22</v>
       </c>
-      <c r="AC7" t="n">
+      <c r="AD7" t="n">
         <v>2.3</v>
       </c>
-      <c r="AD7" t="n">
+      <c r="AE7" t="n">
         <v>1.6</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>Example Firm</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
           <t>MedTech Innovations</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>Fund III</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>Healthcare</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>Western Europe</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>Partially Realized</t>
         </is>
       </c>
-      <c r="F8" s="3" t="inlineStr">
+      <c r="G8" s="3" t="inlineStr">
         <is>
           <t>IPO (Partial Exit)</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="H8" t="inlineStr">
         <is>
           <t>A. Morgan</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="I8" t="inlineStr">
         <is>
           <t>Preferred Equity</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="J8" t="inlineStr">
         <is>
           <t>Growth Buyout</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="K8" t="inlineStr">
         <is>
           <t>Limited Auction</t>
         </is>
       </c>
-      <c r="K8" s="4" t="n">
+      <c r="L8" s="4" t="n">
         <v>43709</v>
       </c>
-      <c r="L8" t="n">
+      <c r="M8" t="n">
         <v>2019</v>
       </c>
-      <c r="N8" t="n">
+      <c r="O8" t="n">
         <v>65</v>
       </c>
-      <c r="O8" t="n">
+      <c r="P8" t="n">
         <v>0.27</v>
       </c>
-      <c r="P8" t="n">
+      <c r="Q8" t="n">
         <v>55</v>
       </c>
-      <c r="Q8" t="n">
+      <c r="R8" t="n">
         <v>10</v>
       </c>
-      <c r="R8" t="n">
+      <c r="S8" t="n">
         <v>160</v>
       </c>
-      <c r="S8" t="n">
+      <c r="T8" t="n">
         <v>45</v>
       </c>
-      <c r="T8" t="n">
+      <c r="U8" t="n">
         <v>110</v>
       </c>
-      <c r="U8" t="n">
+      <c r="V8" t="n">
         <v>28</v>
       </c>
-      <c r="V8" t="n">
+      <c r="W8" t="n">
         <v>390</v>
       </c>
-      <c r="W8" t="n">
+      <c r="X8" t="n">
         <v>50</v>
       </c>
-      <c r="X8" t="n">
+      <c r="Y8" t="n">
         <v>40</v>
       </c>
-      <c r="Y8" t="n">
+      <c r="Z8" t="n">
         <v>82</v>
       </c>
-      <c r="Z8" t="n">
+      <c r="AA8" t="n">
         <v>0.16</v>
       </c>
-      <c r="AA8" t="n">
+      <c r="AB8" t="n">
         <v>620</v>
       </c>
-      <c r="AB8" t="n">
+      <c r="AC8" t="n">
         <v>0.2</v>
       </c>
-      <c r="AC8" t="n">
+      <c r="AD8" t="n">
         <v>2</v>
       </c>
-      <c r="AD8" t="n">
+      <c r="AE8" t="n">
         <v>1.4</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>Example Firm</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
           <t>DataForge AI</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>Fund IV</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>Technology</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>US</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="F9" t="inlineStr">
         <is>
           <t>Unrealized</t>
         </is>
       </c>
-      <c r="F9" s="3" t="inlineStr">
+      <c r="G9" s="3" t="inlineStr">
         <is>
           <t>Unrealized / N.A.</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="H9" t="inlineStr">
         <is>
           <t>S. Nguyen</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="I9" t="inlineStr">
         <is>
           <t>Preferred Equity</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="J9" t="inlineStr">
         <is>
           <t>Platform</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr">
+      <c r="K9" t="inlineStr">
         <is>
           <t>Proprietary</t>
         </is>
       </c>
-      <c r="K9" s="4" t="n">
+      <c r="L9" s="4" t="n">
         <v>44256</v>
       </c>
-      <c r="L9" t="n">
+      <c r="M9" t="n">
         <v>2021</v>
       </c>
-      <c r="N9" t="n">
+      <c r="O9" t="n">
         <v>100</v>
       </c>
-      <c r="O9" t="n">
+      <c r="P9" t="n">
         <v>0.29</v>
       </c>
-      <c r="P9" t="n">
+      <c r="Q9" t="n">
         <v>30</v>
       </c>
-      <c r="Q9" t="n">
+      <c r="R9" t="n">
         <v>5</v>
       </c>
-      <c r="R9" t="n">
+      <c r="S9" t="n">
         <v>150</v>
       </c>
-      <c r="S9" t="n">
+      <c r="T9" t="n">
         <v>20</v>
       </c>
-      <c r="T9" t="n">
+      <c r="U9" t="n">
         <v>85</v>
       </c>
-      <c r="U9" t="n">
+      <c r="V9" t="n">
         <v>22</v>
       </c>
-      <c r="V9" t="n">
+      <c r="W9" t="n">
         <v>400</v>
       </c>
-      <c r="W9" t="n">
+      <c r="X9" t="n">
         <v>35</v>
       </c>
-      <c r="X9" t="n">
+      <c r="Y9" t="n">
         <v>0</v>
       </c>
-      <c r="Y9" t="n">
+      <c r="Z9" t="n">
         <v>195</v>
       </c>
-      <c r="Z9" t="n">
+      <c r="AA9" t="n">
         <v>0.15</v>
       </c>
-      <c r="AA9" t="n">
+      <c r="AB9" t="n">
         <v>710</v>
       </c>
-      <c r="AB9" t="n">
+      <c r="AC9" t="n">
         <v>0.22</v>
       </c>
-      <c r="AC9" t="n">
+      <c r="AD9" t="n">
         <v>2.3</v>
       </c>
-      <c r="AD9" t="n">
+      <c r="AE9" t="n">
         <v>1.6</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>Example Firm</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
           <t>GreenField Energy</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>Fund IV</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="D10" t="inlineStr">
         <is>
           <t>Energy</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>Canada</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="F10" t="inlineStr">
         <is>
           <t>Unrealized</t>
         </is>
       </c>
-      <c r="F10" s="3" t="inlineStr">
+      <c r="G10" s="3" t="inlineStr">
         <is>
           <t>Unrealized / N.A.</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="H10" t="inlineStr">
         <is>
           <t>R. Patel</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
+      <c r="I10" t="inlineStr">
         <is>
           <t>Structured Equity</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
+      <c r="J10" t="inlineStr">
         <is>
           <t>Platform</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr">
+      <c r="K10" t="inlineStr">
         <is>
           <t>Bilateral</t>
         </is>
       </c>
-      <c r="K10" s="4" t="n">
+      <c r="L10" s="4" t="n">
         <v>44576</v>
       </c>
-      <c r="L10" t="n">
+      <c r="M10" t="n">
         <v>2022</v>
       </c>
-      <c r="N10" t="n">
+      <c r="O10" t="n">
         <v>70</v>
       </c>
-      <c r="O10" t="n">
+      <c r="P10" t="n">
         <v>0.24</v>
       </c>
-      <c r="P10" t="n">
+      <c r="Q10" t="n">
         <v>90</v>
       </c>
-      <c r="Q10" t="n">
+      <c r="R10" t="n">
         <v>18</v>
       </c>
-      <c r="R10" t="n">
+      <c r="S10" t="n">
         <v>210</v>
       </c>
-      <c r="S10" t="n">
+      <c r="T10" t="n">
         <v>55</v>
       </c>
-      <c r="T10" t="n">
+      <c r="U10" t="n">
         <v>140</v>
       </c>
-      <c r="U10" t="n">
+      <c r="V10" t="n">
         <v>30</v>
       </c>
-      <c r="V10" t="n">
+      <c r="W10" t="n">
         <v>350</v>
       </c>
-      <c r="W10" t="n">
+      <c r="X10" t="n">
         <v>60</v>
       </c>
-      <c r="X10" t="n">
+      <c r="Y10" t="n">
         <v>0</v>
       </c>
-      <c r="Y10" t="n">
+      <c r="Z10" t="n">
         <v>84</v>
       </c>
-      <c r="Z10" t="n">
+      <c r="AA10" t="n">
         <v>0.12</v>
       </c>
-      <c r="AA10" t="n">
+      <c r="AB10" t="n">
         <v>710</v>
       </c>
-      <c r="AB10" t="n">
+      <c r="AC10" t="n">
         <v>0.22</v>
       </c>
-      <c r="AC10" t="n">
+      <c r="AD10" t="n">
         <v>2.3</v>
       </c>
-      <c r="AD10" t="n">
+      <c r="AE10" t="n">
         <v>1.6</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>Example Firm</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
           <t>Pacific Food Holdings</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>Fund V</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="D11" t="inlineStr">
         <is>
           <t>Consumer</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="E11" t="inlineStr">
         <is>
           <t>APAC</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="F11" t="inlineStr">
         <is>
           <t>Unrealized</t>
         </is>
       </c>
-      <c r="F11" s="3" t="inlineStr">
+      <c r="G11" s="3" t="inlineStr">
         <is>
           <t>Unrealized / N.A.</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
+      <c r="H11" t="inlineStr">
         <is>
           <t>M. Rivera</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="I11" t="inlineStr">
         <is>
           <t>Common Equity</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
+      <c r="J11" t="inlineStr">
         <is>
           <t>Platform</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr">
+      <c r="K11" t="inlineStr">
         <is>
           <t>Broad Auction</t>
         </is>
       </c>
-      <c r="K11" s="4" t="n">
+      <c r="L11" s="4" t="n">
         <v>45078</v>
       </c>
-      <c r="L11" t="n">
+      <c r="M11" t="n">
         <v>2023</v>
       </c>
-      <c r="N11" t="n">
+      <c r="O11" t="n">
         <v>90</v>
       </c>
-      <c r="O11" t="n">
+      <c r="P11" t="n">
         <v>0.37</v>
       </c>
-      <c r="P11" t="n">
+      <c r="Q11" t="n">
         <v>180</v>
       </c>
-      <c r="Q11" t="n">
+      <c r="R11" t="n">
         <v>32</v>
       </c>
-      <c r="R11" t="n">
+      <c r="S11" t="n">
         <v>350</v>
       </c>
-      <c r="S11" t="n">
+      <c r="T11" t="n">
         <v>90</v>
       </c>
-      <c r="T11" t="n">
+      <c r="U11" t="n">
         <v>210</v>
       </c>
-      <c r="U11" t="n">
+      <c r="V11" t="n">
         <v>38</v>
       </c>
-      <c r="V11" t="n">
+      <c r="W11" t="n">
         <v>420</v>
       </c>
-      <c r="W11" t="n">
+      <c r="X11" t="n">
         <v>85</v>
       </c>
-      <c r="X11" t="n">
+      <c r="Y11" t="n">
         <v>0</v>
       </c>
-      <c r="Y11" t="n">
+      <c r="Z11" t="n">
         <v>162</v>
       </c>
-      <c r="Z11" t="n">
+      <c r="AA11" t="n">
         <v>0.1</v>
       </c>
-      <c r="AA11" t="n">
+      <c r="AB11" t="n">
         <v>805</v>
       </c>
-      <c r="AB11" t="n">
+      <c r="AC11" t="n">
         <v>0.24</v>
       </c>
-      <c r="AC11" t="n">
+      <c r="AD11" t="n">
         <v>2.6</v>
       </c>
-      <c r="AD11" t="n">
+      <c r="AE11" t="n">
         <v>1.8</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>Example Firm</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
           <t>Pinnacle Financial Services</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>Fund V</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t>Financial Services</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t>US</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="F12" t="inlineStr">
         <is>
           <t>Unrealized</t>
         </is>
       </c>
-      <c r="F12" s="3" t="inlineStr">
+      <c r="G12" s="3" t="inlineStr">
         <is>
           <t>Unrealized / N.A.</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
+      <c r="H12" t="inlineStr">
         <is>
           <t>T. Brooks</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
+      <c r="I12" t="inlineStr">
         <is>
           <t>Common Equity</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr">
+      <c r="J12" t="inlineStr">
         <is>
           <t>Platform</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr">
+      <c r="K12" t="inlineStr">
         <is>
           <t>Limited Auction</t>
         </is>
       </c>
-      <c r="K12" s="4" t="n">
+      <c r="L12" s="4" t="n">
         <v>45184</v>
       </c>
-      <c r="L12" t="n">
+      <c r="M12" t="n">
         <v>2023</v>
       </c>
-      <c r="N12" t="n">
+      <c r="O12" t="n">
         <v>80</v>
       </c>
-      <c r="O12" t="n">
+      <c r="P12" t="n">
         <v>0.26</v>
       </c>
-      <c r="P12" t="n">
+      <c r="Q12" t="n">
         <v>60</v>
       </c>
-      <c r="Q12" t="n">
+      <c r="R12" t="n">
         <v>15</v>
       </c>
-      <c r="R12" t="n">
+      <c r="S12" t="n">
         <v>175</v>
       </c>
-      <c r="S12" t="n">
+      <c r="T12" t="n">
         <v>30</v>
       </c>
-      <c r="T12" t="n">
+      <c r="U12" t="n">
         <v>72</v>
       </c>
-      <c r="U12" t="n">
+      <c r="V12" t="n">
         <v>19</v>
       </c>
-      <c r="V12" t="n">
+      <c r="W12" t="n">
         <v>220</v>
       </c>
-      <c r="W12" t="n">
+      <c r="X12" t="n">
         <v>28</v>
       </c>
-      <c r="X12" t="n">
+      <c r="Y12" t="n">
         <v>0</v>
       </c>
-      <c r="Y12" t="n">
+      <c r="Z12" t="n">
         <v>104</v>
       </c>
-      <c r="Z12" t="n">
+      <c r="AA12" t="n">
         <v>0.08</v>
       </c>
-      <c r="AA12" t="n">
+      <c r="AB12" t="n">
         <v>805</v>
       </c>
-      <c r="AB12" t="n">
+      <c r="AC12" t="n">
         <v>0.24</v>
       </c>
-      <c r="AC12" t="n">
+      <c r="AD12" t="n">
         <v>2.6</v>
       </c>
-      <c r="AD12" t="n">
+      <c r="AE12" t="n">
         <v>1.8</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
+          <t>Example Firm</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
           <t>CyberShield Security</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>Fund V</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="D13" t="inlineStr">
         <is>
           <t>Technology</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="E13" t="inlineStr">
         <is>
           <t>Europe</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="F13" t="inlineStr">
         <is>
           <t>Unrealized</t>
         </is>
       </c>
-      <c r="F13" s="3" t="inlineStr">
+      <c r="G13" s="3" t="inlineStr">
         <is>
           <t>Unrealized / N.A.</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
+      <c r="H13" t="inlineStr">
         <is>
           <t>S. Nguyen</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
+      <c r="I13" t="inlineStr">
         <is>
           <t>Preferred Equity</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr">
+      <c r="J13" t="inlineStr">
         <is>
           <t>Growth Buyout</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr">
+      <c r="K13" t="inlineStr">
         <is>
           <t>Proprietary</t>
         </is>
       </c>
-      <c r="K13" s="4" t="n">
+      <c r="L13" s="4" t="n">
         <v>45323</v>
       </c>
-      <c r="L13" t="n">
+      <c r="M13" t="n">
         <v>2024</v>
       </c>
-      <c r="N13" t="n">
+      <c r="O13" t="n">
         <v>110</v>
       </c>
-      <c r="O13" t="n">
+      <c r="P13" t="n">
         <v>0.21</v>
       </c>
-      <c r="P13" t="n">
+      <c r="Q13" t="n">
         <v>25</v>
       </c>
-      <c r="Q13" t="n">
+      <c r="R13" t="n">
         <v>3</v>
       </c>
-      <c r="R13" t="n">
+      <c r="S13" t="n">
         <v>120</v>
       </c>
-      <c r="S13" t="n">
+      <c r="T13" t="n">
         <v>15</v>
       </c>
-      <c r="T13" t="n">
+      <c r="U13" t="n">
         <v>35</v>
       </c>
-      <c r="U13" t="n">
+      <c r="V13" t="n">
         <v>6</v>
       </c>
-      <c r="V13" t="n">
+      <c r="W13" t="n">
         <v>180</v>
       </c>
-      <c r="W13" t="n">
+      <c r="X13" t="n">
         <v>18</v>
       </c>
-      <c r="X13" t="n">
+      <c r="Y13" t="n">
         <v>0</v>
       </c>
-      <c r="Y13" t="n">
+      <c r="Z13" t="n">
         <v>176</v>
       </c>
-      <c r="AA13" t="n">
+      <c r="AB13" t="n">
         <v>805</v>
       </c>
-      <c r="AB13" t="n">
+      <c r="AC13" t="n">
         <v>0.24</v>
       </c>
-      <c r="AC13" t="n">
+      <c r="AD13" t="n">
         <v>2.6</v>
       </c>
-      <c r="AD13" t="n">
+      <c r="AE13" t="n">
         <v>1.8</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add firm-level currency support across upload, UI, and PDF
</commit_message>
<xml_diff>
--- a/PE_Fund_Data_Template.xlsx
+++ b/PE_Fund_Data_Template.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE13"/>
+  <dimension ref="A1:AF13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -444,152 +444,157 @@
           <t>Firm Name</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Firm Currency</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Company Name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Fund</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Sector</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Geography</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Exit Type</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Lead Partner</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Security Type</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Deal Type</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Entry Channel</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Investment Date</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Year Invested</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Exit Date</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Equity Invested</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Ownership %</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Entry Revenue</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Entry EBITDA</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Entry EV</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Entry Net Debt</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Exit Revenue</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>Exit EBITDA</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>Exit EV</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>Exit Net Debt</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>Realized Value</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>Unrealized Value</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>IRR</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>Fund Size</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>Net IRR</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>Net MOIC</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>DPI</t>
         </is>
@@ -603,112 +608,117 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
           <t>Apex Healthcare Solutions</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>Fund III</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>Healthcare</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>US</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>Fully Realized</t>
         </is>
       </c>
-      <c r="G2" s="3" t="inlineStr">
+      <c r="H2" s="3" t="inlineStr">
         <is>
           <t>Strategic Sale</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>A. Morgan</t>
         </is>
       </c>
-      <c r="I2" s="3" t="inlineStr">
+      <c r="J2" s="3" t="inlineStr">
         <is>
           <t>Common Equity</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>Platform</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>Proprietary</t>
         </is>
       </c>
-      <c r="L2" s="4" t="n">
+      <c r="M2" s="4" t="n">
         <v>43174</v>
       </c>
-      <c r="M2" t="n">
+      <c r="N2" t="n">
         <v>2018</v>
       </c>
-      <c r="N2" s="4" t="n">
+      <c r="O2" s="4" t="n">
         <v>45107</v>
       </c>
-      <c r="O2" t="n">
+      <c r="P2" t="n">
         <v>75</v>
       </c>
-      <c r="P2" t="n">
+      <c r="Q2" t="n">
         <v>0.42</v>
       </c>
-      <c r="Q2" t="n">
+      <c r="R2" t="n">
         <v>120</v>
       </c>
-      <c r="R2" t="n">
+      <c r="S2" t="n">
         <v>28</v>
       </c>
-      <c r="S2" t="n">
+      <c r="T2" t="n">
         <v>310</v>
       </c>
-      <c r="T2" t="n">
+      <c r="U2" t="n">
         <v>85</v>
       </c>
-      <c r="U2" t="n">
+      <c r="V2" t="n">
         <v>245</v>
       </c>
-      <c r="V2" t="n">
+      <c r="W2" t="n">
         <v>62</v>
       </c>
-      <c r="W2" t="n">
+      <c r="X2" t="n">
         <v>720</v>
       </c>
-      <c r="X2" t="n">
+      <c r="Y2" t="n">
         <v>95</v>
       </c>
-      <c r="Y2" t="n">
+      <c r="Z2" t="n">
         <v>170</v>
       </c>
-      <c r="Z2" t="n">
+      <c r="AA2" t="n">
         <v>0</v>
       </c>
-      <c r="AA2" t="n">
+      <c r="AB2" t="n">
         <v>0.28</v>
       </c>
-      <c r="AB2" t="n">
+      <c r="AC2" t="n">
         <v>620</v>
       </c>
-      <c r="AC2" t="n">
+      <c r="AD2" t="n">
         <v>0.2</v>
       </c>
-      <c r="AD2" t="n">
+      <c r="AE2" t="n">
         <v>2</v>
       </c>
-      <c r="AE2" t="n">
+      <c r="AF2" t="n">
         <v>1.4</v>
       </c>
     </row>
@@ -720,112 +730,117 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
           <t>TechVault Software</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>Fund III</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>Technology</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>US</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>Fully Realized</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr">
+      <c r="H3" s="3" t="inlineStr">
         <is>
           <t>Secondary Buyout</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>L. Chen</t>
         </is>
       </c>
-      <c r="I3" s="3" t="inlineStr">
+      <c r="J3" s="3" t="inlineStr">
         <is>
           <t>Preferred Equity</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>Platform</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>Limited Auction</t>
         </is>
       </c>
-      <c r="L3" s="4" t="n">
+      <c r="M3" s="4" t="n">
         <v>43475</v>
       </c>
-      <c r="M3" t="n">
+      <c r="N3" t="n">
         <v>2019</v>
       </c>
-      <c r="N3" s="4" t="n">
+      <c r="O3" s="4" t="n">
         <v>45397</v>
       </c>
-      <c r="O3" t="n">
+      <c r="P3" t="n">
         <v>50</v>
       </c>
-      <c r="P3" t="n">
+      <c r="Q3" t="n">
         <v>0.35</v>
       </c>
-      <c r="Q3" t="n">
+      <c r="R3" t="n">
         <v>80</v>
       </c>
-      <c r="R3" t="n">
+      <c r="S3" t="n">
         <v>18</v>
       </c>
-      <c r="S3" t="n">
+      <c r="T3" t="n">
         <v>225</v>
       </c>
-      <c r="T3" t="n">
+      <c r="U3" t="n">
         <v>60</v>
       </c>
-      <c r="U3" t="n">
+      <c r="V3" t="n">
         <v>160</v>
       </c>
-      <c r="V3" t="n">
+      <c r="W3" t="n">
         <v>45</v>
       </c>
-      <c r="W3" t="n">
+      <c r="X3" t="n">
         <v>540</v>
       </c>
-      <c r="X3" t="n">
+      <c r="Y3" t="n">
         <v>70</v>
       </c>
-      <c r="Y3" t="n">
+      <c r="Z3" t="n">
         <v>130</v>
       </c>
-      <c r="Z3" t="n">
+      <c r="AA3" t="n">
         <v>0</v>
       </c>
-      <c r="AA3" t="n">
+      <c r="AB3" t="n">
         <v>0.24</v>
       </c>
-      <c r="AB3" t="n">
+      <c r="AC3" t="n">
         <v>620</v>
       </c>
-      <c r="AC3" t="n">
+      <c r="AD3" t="n">
         <v>0.2</v>
       </c>
-      <c r="AD3" t="n">
+      <c r="AE3" t="n">
         <v>2</v>
       </c>
-      <c r="AE3" t="n">
+      <c r="AF3" t="n">
         <v>1.4</v>
       </c>
     </row>
@@ -837,112 +852,117 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
           <t>National Logistics Group</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>Fund II</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>Industrials</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>Western Europe</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>Fully Realized</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="H4" s="3" t="inlineStr">
         <is>
           <t>Strategic Sale</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>R. Patel</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="J4" s="3" t="inlineStr">
         <is>
           <t>Common Equity</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>Carve-out</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>Broad Auction</t>
         </is>
       </c>
-      <c r="L4" s="4" t="n">
+      <c r="M4" s="4" t="n">
         <v>42887</v>
       </c>
-      <c r="M4" t="n">
+      <c r="N4" t="n">
         <v>2017</v>
       </c>
-      <c r="N4" s="4" t="n">
+      <c r="O4" s="4" t="n">
         <v>44834</v>
       </c>
-      <c r="O4" t="n">
+      <c r="P4" t="n">
         <v>60</v>
       </c>
-      <c r="P4" t="n">
+      <c r="Q4" t="n">
         <v>0.28</v>
       </c>
-      <c r="Q4" t="n">
+      <c r="R4" t="n">
         <v>200</v>
       </c>
-      <c r="R4" t="n">
+      <c r="S4" t="n">
         <v>35</v>
       </c>
-      <c r="S4" t="n">
+      <c r="T4" t="n">
         <v>380</v>
       </c>
-      <c r="T4" t="n">
+      <c r="U4" t="n">
         <v>120</v>
       </c>
-      <c r="U4" t="n">
+      <c r="V4" t="n">
         <v>310</v>
       </c>
-      <c r="V4" t="n">
+      <c r="W4" t="n">
         <v>58</v>
       </c>
-      <c r="W4" t="n">
+      <c r="X4" t="n">
         <v>620</v>
       </c>
-      <c r="X4" t="n">
+      <c r="Y4" t="n">
         <v>110</v>
       </c>
-      <c r="Y4" t="n">
+      <c r="Z4" t="n">
         <v>118</v>
       </c>
-      <c r="Z4" t="n">
+      <c r="AA4" t="n">
         <v>0</v>
       </c>
-      <c r="AA4" t="n">
+      <c r="AB4" t="n">
         <v>0.2</v>
       </c>
-      <c r="AB4" t="n">
+      <c r="AC4" t="n">
         <v>550</v>
       </c>
-      <c r="AC4" t="n">
+      <c r="AD4" t="n">
         <v>0.18</v>
       </c>
-      <c r="AD4" t="n">
+      <c r="AE4" t="n">
         <v>1.8</v>
       </c>
-      <c r="AE4" t="n">
+      <c r="AF4" t="n">
         <v>1.2</v>
       </c>
     </row>
@@ -954,112 +974,117 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
           <t>Summit Education Partners</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>Fund II</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>Consumer</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>US</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>Fully Realized</t>
         </is>
       </c>
-      <c r="G5" s="3" t="inlineStr">
+      <c r="H5" s="3" t="inlineStr">
         <is>
           <t>Secondary Buyout</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>M. Rivera</t>
         </is>
       </c>
-      <c r="I5" s="3" t="inlineStr">
+      <c r="J5" s="3" t="inlineStr">
         <is>
           <t>Common Equity</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>Platform</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="L5" t="inlineStr">
         <is>
           <t>Proprietary</t>
         </is>
       </c>
-      <c r="L5" s="4" t="n">
+      <c r="M5" s="4" t="n">
         <v>42694</v>
       </c>
-      <c r="M5" t="n">
+      <c r="N5" t="n">
         <v>2016</v>
       </c>
-      <c r="N5" s="4" t="n">
+      <c r="O5" s="4" t="n">
         <v>44270</v>
       </c>
-      <c r="O5" t="n">
+      <c r="P5" t="n">
         <v>40</v>
       </c>
-      <c r="P5" t="n">
+      <c r="Q5" t="n">
         <v>0.31</v>
       </c>
-      <c r="Q5" t="n">
+      <c r="R5" t="n">
         <v>65</v>
       </c>
-      <c r="R5" t="n">
+      <c r="S5" t="n">
         <v>12</v>
       </c>
-      <c r="S5" t="n">
+      <c r="T5" t="n">
         <v>140</v>
       </c>
-      <c r="T5" t="n">
+      <c r="U5" t="n">
         <v>35</v>
       </c>
-      <c r="U5" t="n">
+      <c r="V5" t="n">
         <v>95</v>
       </c>
-      <c r="V5" t="n">
+      <c r="W5" t="n">
         <v>22</v>
       </c>
-      <c r="W5" t="n">
+      <c r="X5" t="n">
         <v>260</v>
       </c>
-      <c r="X5" t="n">
+      <c r="Y5" t="n">
         <v>30</v>
       </c>
-      <c r="Y5" t="n">
+      <c r="Z5" t="n">
         <v>72</v>
       </c>
-      <c r="Z5" t="n">
+      <c r="AA5" t="n">
         <v>0</v>
       </c>
-      <c r="AA5" t="n">
+      <c r="AB5" t="n">
         <v>0.18</v>
       </c>
-      <c r="AB5" t="n">
+      <c r="AC5" t="n">
         <v>550</v>
       </c>
-      <c r="AC5" t="n">
+      <c r="AD5" t="n">
         <v>0.18</v>
       </c>
-      <c r="AD5" t="n">
+      <c r="AE5" t="n">
         <v>1.8</v>
       </c>
-      <c r="AE5" t="n">
+      <c r="AF5" t="n">
         <v>1.2</v>
       </c>
     </row>
@@ -1071,112 +1096,117 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
           <t>BrightPath Retail</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>Fund II</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>Consumer</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>US</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>Fully Realized</t>
         </is>
       </c>
-      <c r="G6" s="3" t="inlineStr">
+      <c r="H6" s="3" t="inlineStr">
         <is>
           <t>Recapitalization</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="I6" t="inlineStr">
         <is>
           <t>T. Brooks</t>
         </is>
       </c>
-      <c r="I6" s="3" t="inlineStr">
+      <c r="J6" s="3" t="inlineStr">
         <is>
           <t>Convertible Preferred</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="K6" t="inlineStr">
         <is>
           <t>Turnaround</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
+      <c r="L6" t="inlineStr">
         <is>
           <t>Broad Auction</t>
         </is>
       </c>
-      <c r="L6" s="4" t="n">
+      <c r="M6" s="4" t="n">
         <v>42826</v>
       </c>
-      <c r="M6" t="n">
+      <c r="N6" t="n">
         <v>2017</v>
       </c>
-      <c r="N6" s="4" t="n">
+      <c r="O6" s="4" t="n">
         <v>44926</v>
       </c>
-      <c r="O6" t="n">
+      <c r="P6" t="n">
         <v>55</v>
       </c>
-      <c r="P6" t="n">
+      <c r="Q6" t="n">
         <v>0.4</v>
       </c>
-      <c r="Q6" t="n">
+      <c r="R6" t="n">
         <v>150</v>
       </c>
-      <c r="R6" t="n">
+      <c r="S6" t="n">
         <v>25</v>
       </c>
-      <c r="S6" t="n">
+      <c r="T6" t="n">
         <v>280</v>
       </c>
-      <c r="T6" t="n">
+      <c r="U6" t="n">
         <v>75</v>
       </c>
-      <c r="U6" t="n">
+      <c r="V6" t="n">
         <v>130</v>
       </c>
-      <c r="V6" t="n">
+      <c r="W6" t="n">
         <v>20</v>
       </c>
-      <c r="W6" t="n">
+      <c r="X6" t="n">
         <v>230</v>
       </c>
-      <c r="X6" t="n">
+      <c r="Y6" t="n">
         <v>80</v>
       </c>
-      <c r="Y6" t="n">
+      <c r="Z6" t="n">
         <v>45</v>
       </c>
-      <c r="Z6" t="n">
+      <c r="AA6" t="n">
         <v>0</v>
       </c>
-      <c r="AA6" t="n">
+      <c r="AB6" t="n">
         <v>-0.03</v>
       </c>
-      <c r="AB6" t="n">
+      <c r="AC6" t="n">
         <v>550</v>
       </c>
-      <c r="AC6" t="n">
+      <c r="AD6" t="n">
         <v>0.18</v>
       </c>
-      <c r="AD6" t="n">
+      <c r="AE6" t="n">
         <v>1.8</v>
       </c>
-      <c r="AE6" t="n">
+      <c r="AF6" t="n">
         <v>1.2</v>
       </c>
     </row>
@@ -1188,112 +1218,117 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
           <t>CloudBridge Analytics</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>Fund IV</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>Technology</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>US</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="G7" t="inlineStr">
         <is>
           <t>Partially Realized</t>
         </is>
       </c>
-      <c r="G7" s="3" t="inlineStr">
+      <c r="H7" s="3" t="inlineStr">
         <is>
           <t>Minority Recap</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="I7" t="inlineStr">
         <is>
           <t>L. Chen</t>
         </is>
       </c>
-      <c r="I7" s="3" t="inlineStr">
+      <c r="J7" s="3" t="inlineStr">
         <is>
           <t>Common Equity</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="K7" t="inlineStr">
         <is>
           <t>Platform</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr">
+      <c r="L7" t="inlineStr">
         <is>
           <t>Proprietary</t>
         </is>
       </c>
-      <c r="L7" s="4" t="n">
+      <c r="M7" s="4" t="n">
         <v>44027</v>
       </c>
-      <c r="M7" t="n">
+      <c r="N7" t="n">
         <v>2020</v>
       </c>
-      <c r="N7" s="4" t="n">
+      <c r="O7" s="4" t="n">
         <v>45505</v>
       </c>
-      <c r="O7" t="n">
+      <c r="P7" t="n">
         <v>85</v>
       </c>
-      <c r="P7" t="n">
+      <c r="Q7" t="n">
         <v>0.33</v>
       </c>
-      <c r="Q7" t="n">
+      <c r="R7" t="n">
         <v>45</v>
       </c>
-      <c r="R7" t="n">
+      <c r="S7" t="n">
         <v>8</v>
       </c>
-      <c r="S7" t="n">
+      <c r="T7" t="n">
         <v>190</v>
       </c>
-      <c r="T7" t="n">
+      <c r="U7" t="n">
         <v>40</v>
       </c>
-      <c r="U7" t="n">
+      <c r="V7" t="n">
         <v>130</v>
       </c>
-      <c r="V7" t="n">
+      <c r="W7" t="n">
         <v>35</v>
       </c>
-      <c r="W7" t="n">
+      <c r="X7" t="n">
         <v>520</v>
       </c>
-      <c r="X7" t="n">
+      <c r="Y7" t="n">
         <v>55</v>
       </c>
-      <c r="Y7" t="n">
+      <c r="Z7" t="n">
         <v>90</v>
       </c>
-      <c r="Z7" t="n">
+      <c r="AA7" t="n">
         <v>75</v>
       </c>
-      <c r="AA7" t="n">
+      <c r="AB7" t="n">
         <v>0.3</v>
       </c>
-      <c r="AB7" t="n">
+      <c r="AC7" t="n">
         <v>710</v>
       </c>
-      <c r="AC7" t="n">
+      <c r="AD7" t="n">
         <v>0.22</v>
       </c>
-      <c r="AD7" t="n">
+      <c r="AE7" t="n">
         <v>2.3</v>
       </c>
-      <c r="AE7" t="n">
+      <c r="AF7" t="n">
         <v>1.6</v>
       </c>
     </row>
@@ -1305,109 +1340,114 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
           <t>MedTech Innovations</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>Fund III</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>Healthcare</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>Western Europe</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t>Partially Realized</t>
         </is>
       </c>
-      <c r="G8" s="3" t="inlineStr">
+      <c r="H8" s="3" t="inlineStr">
         <is>
           <t>IPO (Partial Exit)</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="I8" t="inlineStr">
         <is>
           <t>A. Morgan</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="J8" t="inlineStr">
         <is>
           <t>Preferred Equity</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="K8" t="inlineStr">
         <is>
           <t>Growth Buyout</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr">
+      <c r="L8" t="inlineStr">
         <is>
           <t>Limited Auction</t>
         </is>
       </c>
-      <c r="L8" s="4" t="n">
+      <c r="M8" s="4" t="n">
         <v>43709</v>
       </c>
-      <c r="M8" t="n">
+      <c r="N8" t="n">
         <v>2019</v>
       </c>
-      <c r="O8" t="n">
+      <c r="P8" t="n">
         <v>65</v>
       </c>
-      <c r="P8" t="n">
+      <c r="Q8" t="n">
         <v>0.27</v>
       </c>
-      <c r="Q8" t="n">
+      <c r="R8" t="n">
         <v>55</v>
       </c>
-      <c r="R8" t="n">
+      <c r="S8" t="n">
         <v>10</v>
       </c>
-      <c r="S8" t="n">
+      <c r="T8" t="n">
         <v>160</v>
       </c>
-      <c r="T8" t="n">
+      <c r="U8" t="n">
         <v>45</v>
       </c>
-      <c r="U8" t="n">
+      <c r="V8" t="n">
         <v>110</v>
       </c>
-      <c r="V8" t="n">
+      <c r="W8" t="n">
         <v>28</v>
       </c>
-      <c r="W8" t="n">
+      <c r="X8" t="n">
         <v>390</v>
       </c>
-      <c r="X8" t="n">
+      <c r="Y8" t="n">
         <v>50</v>
       </c>
-      <c r="Y8" t="n">
+      <c r="Z8" t="n">
         <v>40</v>
       </c>
-      <c r="Z8" t="n">
+      <c r="AA8" t="n">
         <v>82</v>
       </c>
-      <c r="AA8" t="n">
+      <c r="AB8" t="n">
         <v>0.16</v>
       </c>
-      <c r="AB8" t="n">
+      <c r="AC8" t="n">
         <v>620</v>
       </c>
-      <c r="AC8" t="n">
+      <c r="AD8" t="n">
         <v>0.2</v>
       </c>
-      <c r="AD8" t="n">
+      <c r="AE8" t="n">
         <v>2</v>
       </c>
-      <c r="AE8" t="n">
+      <c r="AF8" t="n">
         <v>1.4</v>
       </c>
     </row>
@@ -1419,109 +1459,114 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
           <t>DataForge AI</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>Fund IV</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>Technology</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="F9" t="inlineStr">
         <is>
           <t>US</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="G9" t="inlineStr">
         <is>
           <t>Unrealized</t>
         </is>
       </c>
-      <c r="G9" s="3" t="inlineStr">
+      <c r="H9" s="3" t="inlineStr">
         <is>
           <t>Unrealized / N.A.</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="I9" t="inlineStr">
         <is>
           <t>S. Nguyen</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="J9" t="inlineStr">
         <is>
           <t>Preferred Equity</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr">
+      <c r="K9" t="inlineStr">
         <is>
           <t>Platform</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr">
+      <c r="L9" t="inlineStr">
         <is>
           <t>Proprietary</t>
         </is>
       </c>
-      <c r="L9" s="4" t="n">
+      <c r="M9" s="4" t="n">
         <v>44256</v>
       </c>
-      <c r="M9" t="n">
+      <c r="N9" t="n">
         <v>2021</v>
       </c>
-      <c r="O9" t="n">
+      <c r="P9" t="n">
         <v>100</v>
       </c>
-      <c r="P9" t="n">
+      <c r="Q9" t="n">
         <v>0.29</v>
       </c>
-      <c r="Q9" t="n">
+      <c r="R9" t="n">
         <v>30</v>
       </c>
-      <c r="R9" t="n">
+      <c r="S9" t="n">
         <v>5</v>
       </c>
-      <c r="S9" t="n">
+      <c r="T9" t="n">
         <v>150</v>
       </c>
-      <c r="T9" t="n">
+      <c r="U9" t="n">
         <v>20</v>
       </c>
-      <c r="U9" t="n">
+      <c r="V9" t="n">
         <v>85</v>
       </c>
-      <c r="V9" t="n">
+      <c r="W9" t="n">
         <v>22</v>
       </c>
-      <c r="W9" t="n">
+      <c r="X9" t="n">
         <v>400</v>
       </c>
-      <c r="X9" t="n">
+      <c r="Y9" t="n">
         <v>35</v>
       </c>
-      <c r="Y9" t="n">
+      <c r="Z9" t="n">
         <v>0</v>
       </c>
-      <c r="Z9" t="n">
+      <c r="AA9" t="n">
         <v>195</v>
       </c>
-      <c r="AA9" t="n">
+      <c r="AB9" t="n">
         <v>0.15</v>
       </c>
-      <c r="AB9" t="n">
+      <c r="AC9" t="n">
         <v>710</v>
       </c>
-      <c r="AC9" t="n">
+      <c r="AD9" t="n">
         <v>0.22</v>
       </c>
-      <c r="AD9" t="n">
+      <c r="AE9" t="n">
         <v>2.3</v>
       </c>
-      <c r="AE9" t="n">
+      <c r="AF9" t="n">
         <v>1.6</v>
       </c>
     </row>
@@ -1533,109 +1578,114 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
           <t>GreenField Energy</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="D10" t="inlineStr">
         <is>
           <t>Fund IV</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>Energy</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="F10" t="inlineStr">
         <is>
           <t>Canada</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="G10" t="inlineStr">
         <is>
           <t>Unrealized</t>
         </is>
       </c>
-      <c r="G10" s="3" t="inlineStr">
+      <c r="H10" s="3" t="inlineStr">
         <is>
           <t>Unrealized / N.A.</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
+      <c r="I10" t="inlineStr">
         <is>
           <t>R. Patel</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
+      <c r="J10" t="inlineStr">
         <is>
           <t>Structured Equity</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr">
+      <c r="K10" t="inlineStr">
         <is>
           <t>Platform</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr">
+      <c r="L10" t="inlineStr">
         <is>
           <t>Bilateral</t>
         </is>
       </c>
-      <c r="L10" s="4" t="n">
+      <c r="M10" s="4" t="n">
         <v>44576</v>
       </c>
-      <c r="M10" t="n">
+      <c r="N10" t="n">
         <v>2022</v>
       </c>
-      <c r="O10" t="n">
+      <c r="P10" t="n">
         <v>70</v>
       </c>
-      <c r="P10" t="n">
+      <c r="Q10" t="n">
         <v>0.24</v>
       </c>
-      <c r="Q10" t="n">
+      <c r="R10" t="n">
         <v>90</v>
       </c>
-      <c r="R10" t="n">
+      <c r="S10" t="n">
         <v>18</v>
       </c>
-      <c r="S10" t="n">
+      <c r="T10" t="n">
         <v>210</v>
       </c>
-      <c r="T10" t="n">
+      <c r="U10" t="n">
         <v>55</v>
       </c>
-      <c r="U10" t="n">
+      <c r="V10" t="n">
         <v>140</v>
       </c>
-      <c r="V10" t="n">
+      <c r="W10" t="n">
         <v>30</v>
       </c>
-      <c r="W10" t="n">
+      <c r="X10" t="n">
         <v>350</v>
       </c>
-      <c r="X10" t="n">
+      <c r="Y10" t="n">
         <v>60</v>
       </c>
-      <c r="Y10" t="n">
+      <c r="Z10" t="n">
         <v>0</v>
       </c>
-      <c r="Z10" t="n">
+      <c r="AA10" t="n">
         <v>84</v>
       </c>
-      <c r="AA10" t="n">
+      <c r="AB10" t="n">
         <v>0.12</v>
       </c>
-      <c r="AB10" t="n">
+      <c r="AC10" t="n">
         <v>710</v>
       </c>
-      <c r="AC10" t="n">
+      <c r="AD10" t="n">
         <v>0.22</v>
       </c>
-      <c r="AD10" t="n">
+      <c r="AE10" t="n">
         <v>2.3</v>
       </c>
-      <c r="AE10" t="n">
+      <c r="AF10" t="n">
         <v>1.6</v>
       </c>
     </row>
@@ -1647,109 +1697,114 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
           <t>Pacific Food Holdings</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="D11" t="inlineStr">
         <is>
           <t>Fund V</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="E11" t="inlineStr">
         <is>
           <t>Consumer</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="F11" t="inlineStr">
         <is>
           <t>APAC</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="G11" t="inlineStr">
         <is>
           <t>Unrealized</t>
         </is>
       </c>
-      <c r="G11" s="3" t="inlineStr">
+      <c r="H11" s="3" t="inlineStr">
         <is>
           <t>Unrealized / N.A.</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="I11" t="inlineStr">
         <is>
           <t>M. Rivera</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
+      <c r="J11" t="inlineStr">
         <is>
           <t>Common Equity</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr">
+      <c r="K11" t="inlineStr">
         <is>
           <t>Platform</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr">
+      <c r="L11" t="inlineStr">
         <is>
           <t>Broad Auction</t>
         </is>
       </c>
-      <c r="L11" s="4" t="n">
+      <c r="M11" s="4" t="n">
         <v>45078</v>
       </c>
-      <c r="M11" t="n">
+      <c r="N11" t="n">
         <v>2023</v>
       </c>
-      <c r="O11" t="n">
+      <c r="P11" t="n">
         <v>90</v>
       </c>
-      <c r="P11" t="n">
+      <c r="Q11" t="n">
         <v>0.37</v>
       </c>
-      <c r="Q11" t="n">
+      <c r="R11" t="n">
         <v>180</v>
       </c>
-      <c r="R11" t="n">
+      <c r="S11" t="n">
         <v>32</v>
       </c>
-      <c r="S11" t="n">
+      <c r="T11" t="n">
         <v>350</v>
       </c>
-      <c r="T11" t="n">
+      <c r="U11" t="n">
         <v>90</v>
       </c>
-      <c r="U11" t="n">
+      <c r="V11" t="n">
         <v>210</v>
       </c>
-      <c r="V11" t="n">
+      <c r="W11" t="n">
         <v>38</v>
       </c>
-      <c r="W11" t="n">
+      <c r="X11" t="n">
         <v>420</v>
       </c>
-      <c r="X11" t="n">
+      <c r="Y11" t="n">
         <v>85</v>
       </c>
-      <c r="Y11" t="n">
+      <c r="Z11" t="n">
         <v>0</v>
       </c>
-      <c r="Z11" t="n">
+      <c r="AA11" t="n">
         <v>162</v>
       </c>
-      <c r="AA11" t="n">
+      <c r="AB11" t="n">
         <v>0.1</v>
       </c>
-      <c r="AB11" t="n">
+      <c r="AC11" t="n">
         <v>805</v>
       </c>
-      <c r="AC11" t="n">
+      <c r="AD11" t="n">
         <v>0.24</v>
       </c>
-      <c r="AD11" t="n">
+      <c r="AE11" t="n">
         <v>2.6</v>
       </c>
-      <c r="AE11" t="n">
+      <c r="AF11" t="n">
         <v>1.8</v>
       </c>
     </row>
@@ -1761,109 +1816,114 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
           <t>Pinnacle Financial Services</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t>Fund V</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t>Financial Services</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="F12" t="inlineStr">
         <is>
           <t>US</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="G12" t="inlineStr">
         <is>
           <t>Unrealized</t>
         </is>
       </c>
-      <c r="G12" s="3" t="inlineStr">
+      <c r="H12" s="3" t="inlineStr">
         <is>
           <t>Unrealized / N.A.</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
+      <c r="I12" t="inlineStr">
         <is>
           <t>T. Brooks</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr">
+      <c r="J12" t="inlineStr">
         <is>
           <t>Common Equity</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr">
+      <c r="K12" t="inlineStr">
         <is>
           <t>Platform</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr">
+      <c r="L12" t="inlineStr">
         <is>
           <t>Limited Auction</t>
         </is>
       </c>
-      <c r="L12" s="4" t="n">
+      <c r="M12" s="4" t="n">
         <v>45184</v>
       </c>
-      <c r="M12" t="n">
+      <c r="N12" t="n">
         <v>2023</v>
       </c>
-      <c r="O12" t="n">
+      <c r="P12" t="n">
         <v>80</v>
       </c>
-      <c r="P12" t="n">
+      <c r="Q12" t="n">
         <v>0.26</v>
       </c>
-      <c r="Q12" t="n">
+      <c r="R12" t="n">
         <v>60</v>
       </c>
-      <c r="R12" t="n">
+      <c r="S12" t="n">
         <v>15</v>
       </c>
-      <c r="S12" t="n">
+      <c r="T12" t="n">
         <v>175</v>
       </c>
-      <c r="T12" t="n">
+      <c r="U12" t="n">
         <v>30</v>
       </c>
-      <c r="U12" t="n">
+      <c r="V12" t="n">
         <v>72</v>
       </c>
-      <c r="V12" t="n">
+      <c r="W12" t="n">
         <v>19</v>
       </c>
-      <c r="W12" t="n">
+      <c r="X12" t="n">
         <v>220</v>
       </c>
-      <c r="X12" t="n">
+      <c r="Y12" t="n">
         <v>28</v>
       </c>
-      <c r="Y12" t="n">
+      <c r="Z12" t="n">
         <v>0</v>
       </c>
-      <c r="Z12" t="n">
+      <c r="AA12" t="n">
         <v>104</v>
       </c>
-      <c r="AA12" t="n">
+      <c r="AB12" t="n">
         <v>0.08</v>
       </c>
-      <c r="AB12" t="n">
+      <c r="AC12" t="n">
         <v>805</v>
       </c>
-      <c r="AC12" t="n">
+      <c r="AD12" t="n">
         <v>0.24</v>
       </c>
-      <c r="AD12" t="n">
+      <c r="AE12" t="n">
         <v>2.6</v>
       </c>
-      <c r="AE12" t="n">
+      <c r="AF12" t="n">
         <v>1.8</v>
       </c>
     </row>
@@ -1875,106 +1935,111 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
           <t>CyberShield Security</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="D13" t="inlineStr">
         <is>
           <t>Fund V</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="E13" t="inlineStr">
         <is>
           <t>Technology</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="F13" t="inlineStr">
         <is>
           <t>Europe</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="G13" t="inlineStr">
         <is>
           <t>Unrealized</t>
         </is>
       </c>
-      <c r="G13" s="3" t="inlineStr">
+      <c r="H13" s="3" t="inlineStr">
         <is>
           <t>Unrealized / N.A.</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
+      <c r="I13" t="inlineStr">
         <is>
           <t>S. Nguyen</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr">
+      <c r="J13" t="inlineStr">
         <is>
           <t>Preferred Equity</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr">
+      <c r="K13" t="inlineStr">
         <is>
           <t>Growth Buyout</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr">
+      <c r="L13" t="inlineStr">
         <is>
           <t>Proprietary</t>
         </is>
       </c>
-      <c r="L13" s="4" t="n">
+      <c r="M13" s="4" t="n">
         <v>45323</v>
       </c>
-      <c r="M13" t="n">
+      <c r="N13" t="n">
         <v>2024</v>
       </c>
-      <c r="O13" t="n">
+      <c r="P13" t="n">
         <v>110</v>
       </c>
-      <c r="P13" t="n">
+      <c r="Q13" t="n">
         <v>0.21</v>
       </c>
-      <c r="Q13" t="n">
+      <c r="R13" t="n">
         <v>25</v>
       </c>
-      <c r="R13" t="n">
+      <c r="S13" t="n">
         <v>3</v>
       </c>
-      <c r="S13" t="n">
+      <c r="T13" t="n">
         <v>120</v>
       </c>
-      <c r="T13" t="n">
+      <c r="U13" t="n">
         <v>15</v>
       </c>
-      <c r="U13" t="n">
+      <c r="V13" t="n">
         <v>35</v>
       </c>
-      <c r="V13" t="n">
+      <c r="W13" t="n">
         <v>6</v>
       </c>
-      <c r="W13" t="n">
+      <c r="X13" t="n">
         <v>180</v>
       </c>
-      <c r="X13" t="n">
+      <c r="Y13" t="n">
         <v>18</v>
       </c>
-      <c r="Y13" t="n">
+      <c r="Z13" t="n">
         <v>0</v>
       </c>
-      <c r="Z13" t="n">
+      <c r="AA13" t="n">
         <v>176</v>
       </c>
-      <c r="AB13" t="n">
+      <c r="AC13" t="n">
         <v>805</v>
       </c>
-      <c r="AC13" t="n">
+      <c r="AD13" t="n">
         <v>0.24</v>
       </c>
-      <c r="AD13" t="n">
+      <c r="AE13" t="n">
         <v>2.6</v>
       </c>
-      <c r="AE13" t="n">
+      <c r="AF13" t="n">
         <v>1.8</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add upload-level As Of Date flow across dashboard and analysis
</commit_message>
<xml_diff>
--- a/PE_Fund_Data_Template.xlsx
+++ b/PE_Fund_Data_Template.xlsx
@@ -20,9 +20,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
     <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="2">
     <font>
@@ -62,7 +63,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
@@ -70,6 +71,7 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -435,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF13"/>
+  <dimension ref="A1:AG13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -514,87 +516,92 @@
           <t>Exit Date</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>As Of Date</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Equity Invested</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Ownership %</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Entry Revenue</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Entry EBITDA</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Entry EV</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Entry Net Debt</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>Exit Revenue</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>Exit EBITDA</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>Exit EV</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>Exit Net Debt</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>Realized Value</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>Unrealized Value</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>IRR</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>Fund Size</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>Net IRR</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>Net MOIC</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>DPI</t>
         </is>
@@ -670,55 +677,58 @@
       <c r="O2" s="4" t="n">
         <v>45107</v>
       </c>
-      <c r="P2" t="n">
+      <c r="P2" s="5" t="n">
+        <v>46022</v>
+      </c>
+      <c r="Q2" t="n">
         <v>75</v>
       </c>
-      <c r="Q2" t="n">
+      <c r="R2" t="n">
         <v>0.42</v>
       </c>
-      <c r="R2" t="n">
+      <c r="S2" t="n">
         <v>120</v>
       </c>
-      <c r="S2" t="n">
+      <c r="T2" t="n">
         <v>28</v>
       </c>
-      <c r="T2" t="n">
+      <c r="U2" t="n">
         <v>310</v>
       </c>
-      <c r="U2" t="n">
+      <c r="V2" t="n">
         <v>85</v>
       </c>
-      <c r="V2" t="n">
+      <c r="W2" t="n">
         <v>245</v>
       </c>
-      <c r="W2" t="n">
+      <c r="X2" t="n">
         <v>62</v>
       </c>
-      <c r="X2" t="n">
+      <c r="Y2" t="n">
         <v>720</v>
       </c>
-      <c r="Y2" t="n">
+      <c r="Z2" t="n">
         <v>95</v>
       </c>
-      <c r="Z2" t="n">
+      <c r="AA2" t="n">
         <v>170</v>
       </c>
-      <c r="AA2" t="n">
+      <c r="AB2" t="n">
         <v>0</v>
       </c>
-      <c r="AB2" t="n">
+      <c r="AC2" t="n">
         <v>0.28</v>
       </c>
-      <c r="AC2" t="n">
+      <c r="AD2" t="n">
         <v>620</v>
       </c>
-      <c r="AD2" t="n">
+      <c r="AE2" t="n">
         <v>0.2</v>
       </c>
-      <c r="AE2" t="n">
+      <c r="AF2" t="n">
         <v>2</v>
       </c>
-      <c r="AF2" t="n">
+      <c r="AG2" t="n">
         <v>1.4</v>
       </c>
     </row>
@@ -792,55 +802,58 @@
       <c r="O3" s="4" t="n">
         <v>45397</v>
       </c>
-      <c r="P3" t="n">
+      <c r="P3" s="5" t="n">
+        <v>46022</v>
+      </c>
+      <c r="Q3" t="n">
         <v>50</v>
       </c>
-      <c r="Q3" t="n">
+      <c r="R3" t="n">
         <v>0.35</v>
       </c>
-      <c r="R3" t="n">
+      <c r="S3" t="n">
         <v>80</v>
       </c>
-      <c r="S3" t="n">
+      <c r="T3" t="n">
         <v>18</v>
       </c>
-      <c r="T3" t="n">
+      <c r="U3" t="n">
         <v>225</v>
       </c>
-      <c r="U3" t="n">
+      <c r="V3" t="n">
         <v>60</v>
       </c>
-      <c r="V3" t="n">
+      <c r="W3" t="n">
         <v>160</v>
       </c>
-      <c r="W3" t="n">
+      <c r="X3" t="n">
         <v>45</v>
       </c>
-      <c r="X3" t="n">
+      <c r="Y3" t="n">
         <v>540</v>
       </c>
-      <c r="Y3" t="n">
+      <c r="Z3" t="n">
         <v>70</v>
       </c>
-      <c r="Z3" t="n">
+      <c r="AA3" t="n">
         <v>130</v>
       </c>
-      <c r="AA3" t="n">
+      <c r="AB3" t="n">
         <v>0</v>
       </c>
-      <c r="AB3" t="n">
+      <c r="AC3" t="n">
         <v>0.24</v>
       </c>
-      <c r="AC3" t="n">
+      <c r="AD3" t="n">
         <v>620</v>
       </c>
-      <c r="AD3" t="n">
+      <c r="AE3" t="n">
         <v>0.2</v>
       </c>
-      <c r="AE3" t="n">
+      <c r="AF3" t="n">
         <v>2</v>
       </c>
-      <c r="AF3" t="n">
+      <c r="AG3" t="n">
         <v>1.4</v>
       </c>
     </row>
@@ -914,55 +927,58 @@
       <c r="O4" s="4" t="n">
         <v>44834</v>
       </c>
-      <c r="P4" t="n">
+      <c r="P4" s="5" t="n">
+        <v>46022</v>
+      </c>
+      <c r="Q4" t="n">
         <v>60</v>
       </c>
-      <c r="Q4" t="n">
+      <c r="R4" t="n">
         <v>0.28</v>
       </c>
-      <c r="R4" t="n">
+      <c r="S4" t="n">
         <v>200</v>
       </c>
-      <c r="S4" t="n">
+      <c r="T4" t="n">
         <v>35</v>
       </c>
-      <c r="T4" t="n">
+      <c r="U4" t="n">
         <v>380</v>
       </c>
-      <c r="U4" t="n">
+      <c r="V4" t="n">
         <v>120</v>
       </c>
-      <c r="V4" t="n">
+      <c r="W4" t="n">
         <v>310</v>
       </c>
-      <c r="W4" t="n">
+      <c r="X4" t="n">
         <v>58</v>
       </c>
-      <c r="X4" t="n">
+      <c r="Y4" t="n">
         <v>620</v>
       </c>
-      <c r="Y4" t="n">
+      <c r="Z4" t="n">
         <v>110</v>
       </c>
-      <c r="Z4" t="n">
+      <c r="AA4" t="n">
         <v>118</v>
       </c>
-      <c r="AA4" t="n">
+      <c r="AB4" t="n">
         <v>0</v>
       </c>
-      <c r="AB4" t="n">
+      <c r="AC4" t="n">
         <v>0.2</v>
       </c>
-      <c r="AC4" t="n">
+      <c r="AD4" t="n">
         <v>550</v>
       </c>
-      <c r="AD4" t="n">
+      <c r="AE4" t="n">
         <v>0.18</v>
       </c>
-      <c r="AE4" t="n">
+      <c r="AF4" t="n">
         <v>1.8</v>
       </c>
-      <c r="AF4" t="n">
+      <c r="AG4" t="n">
         <v>1.2</v>
       </c>
     </row>
@@ -1036,55 +1052,58 @@
       <c r="O5" s="4" t="n">
         <v>44270</v>
       </c>
-      <c r="P5" t="n">
+      <c r="P5" s="5" t="n">
+        <v>46022</v>
+      </c>
+      <c r="Q5" t="n">
         <v>40</v>
       </c>
-      <c r="Q5" t="n">
+      <c r="R5" t="n">
         <v>0.31</v>
       </c>
-      <c r="R5" t="n">
+      <c r="S5" t="n">
         <v>65</v>
       </c>
-      <c r="S5" t="n">
+      <c r="T5" t="n">
         <v>12</v>
       </c>
-      <c r="T5" t="n">
+      <c r="U5" t="n">
         <v>140</v>
       </c>
-      <c r="U5" t="n">
+      <c r="V5" t="n">
         <v>35</v>
       </c>
-      <c r="V5" t="n">
+      <c r="W5" t="n">
         <v>95</v>
       </c>
-      <c r="W5" t="n">
+      <c r="X5" t="n">
         <v>22</v>
       </c>
-      <c r="X5" t="n">
+      <c r="Y5" t="n">
         <v>260</v>
       </c>
-      <c r="Y5" t="n">
+      <c r="Z5" t="n">
         <v>30</v>
       </c>
-      <c r="Z5" t="n">
+      <c r="AA5" t="n">
         <v>72</v>
       </c>
-      <c r="AA5" t="n">
+      <c r="AB5" t="n">
         <v>0</v>
       </c>
-      <c r="AB5" t="n">
+      <c r="AC5" t="n">
         <v>0.18</v>
       </c>
-      <c r="AC5" t="n">
+      <c r="AD5" t="n">
         <v>550</v>
       </c>
-      <c r="AD5" t="n">
+      <c r="AE5" t="n">
         <v>0.18</v>
       </c>
-      <c r="AE5" t="n">
+      <c r="AF5" t="n">
         <v>1.8</v>
       </c>
-      <c r="AF5" t="n">
+      <c r="AG5" t="n">
         <v>1.2</v>
       </c>
     </row>
@@ -1158,55 +1177,58 @@
       <c r="O6" s="4" t="n">
         <v>44926</v>
       </c>
-      <c r="P6" t="n">
+      <c r="P6" s="5" t="n">
+        <v>46022</v>
+      </c>
+      <c r="Q6" t="n">
         <v>55</v>
       </c>
-      <c r="Q6" t="n">
+      <c r="R6" t="n">
         <v>0.4</v>
       </c>
-      <c r="R6" t="n">
+      <c r="S6" t="n">
         <v>150</v>
       </c>
-      <c r="S6" t="n">
+      <c r="T6" t="n">
         <v>25</v>
       </c>
-      <c r="T6" t="n">
+      <c r="U6" t="n">
         <v>280</v>
       </c>
-      <c r="U6" t="n">
+      <c r="V6" t="n">
         <v>75</v>
       </c>
-      <c r="V6" t="n">
+      <c r="W6" t="n">
         <v>130</v>
       </c>
-      <c r="W6" t="n">
+      <c r="X6" t="n">
         <v>20</v>
       </c>
-      <c r="X6" t="n">
+      <c r="Y6" t="n">
         <v>230</v>
       </c>
-      <c r="Y6" t="n">
+      <c r="Z6" t="n">
         <v>80</v>
       </c>
-      <c r="Z6" t="n">
+      <c r="AA6" t="n">
         <v>45</v>
       </c>
-      <c r="AA6" t="n">
+      <c r="AB6" t="n">
         <v>0</v>
       </c>
-      <c r="AB6" t="n">
+      <c r="AC6" t="n">
         <v>-0.03</v>
       </c>
-      <c r="AC6" t="n">
+      <c r="AD6" t="n">
         <v>550</v>
       </c>
-      <c r="AD6" t="n">
+      <c r="AE6" t="n">
         <v>0.18</v>
       </c>
-      <c r="AE6" t="n">
+      <c r="AF6" t="n">
         <v>1.8</v>
       </c>
-      <c r="AF6" t="n">
+      <c r="AG6" t="n">
         <v>1.2</v>
       </c>
     </row>
@@ -1280,55 +1302,58 @@
       <c r="O7" s="4" t="n">
         <v>45505</v>
       </c>
-      <c r="P7" t="n">
+      <c r="P7" s="5" t="n">
+        <v>46022</v>
+      </c>
+      <c r="Q7" t="n">
         <v>85</v>
       </c>
-      <c r="Q7" t="n">
+      <c r="R7" t="n">
         <v>0.33</v>
       </c>
-      <c r="R7" t="n">
+      <c r="S7" t="n">
         <v>45</v>
       </c>
-      <c r="S7" t="n">
+      <c r="T7" t="n">
         <v>8</v>
       </c>
-      <c r="T7" t="n">
+      <c r="U7" t="n">
         <v>190</v>
       </c>
-      <c r="U7" t="n">
+      <c r="V7" t="n">
         <v>40</v>
       </c>
-      <c r="V7" t="n">
+      <c r="W7" t="n">
         <v>130</v>
       </c>
-      <c r="W7" t="n">
+      <c r="X7" t="n">
         <v>35</v>
       </c>
-      <c r="X7" t="n">
+      <c r="Y7" t="n">
         <v>520</v>
       </c>
-      <c r="Y7" t="n">
+      <c r="Z7" t="n">
         <v>55</v>
       </c>
-      <c r="Z7" t="n">
+      <c r="AA7" t="n">
         <v>90</v>
       </c>
-      <c r="AA7" t="n">
+      <c r="AB7" t="n">
         <v>75</v>
       </c>
-      <c r="AB7" t="n">
+      <c r="AC7" t="n">
         <v>0.3</v>
       </c>
-      <c r="AC7" t="n">
+      <c r="AD7" t="n">
         <v>710</v>
       </c>
-      <c r="AD7" t="n">
+      <c r="AE7" t="n">
         <v>0.22</v>
       </c>
-      <c r="AE7" t="n">
+      <c r="AF7" t="n">
         <v>2.3</v>
       </c>
-      <c r="AF7" t="n">
+      <c r="AG7" t="n">
         <v>1.6</v>
       </c>
     </row>
@@ -1399,55 +1424,58 @@
       <c r="N8" t="n">
         <v>2019</v>
       </c>
-      <c r="P8" t="n">
+      <c r="P8" s="5" t="n">
+        <v>46022</v>
+      </c>
+      <c r="Q8" t="n">
         <v>65</v>
       </c>
-      <c r="Q8" t="n">
+      <c r="R8" t="n">
         <v>0.27</v>
       </c>
-      <c r="R8" t="n">
+      <c r="S8" t="n">
         <v>55</v>
       </c>
-      <c r="S8" t="n">
+      <c r="T8" t="n">
         <v>10</v>
       </c>
-      <c r="T8" t="n">
+      <c r="U8" t="n">
         <v>160</v>
       </c>
-      <c r="U8" t="n">
+      <c r="V8" t="n">
         <v>45</v>
       </c>
-      <c r="V8" t="n">
+      <c r="W8" t="n">
         <v>110</v>
       </c>
-      <c r="W8" t="n">
+      <c r="X8" t="n">
         <v>28</v>
       </c>
-      <c r="X8" t="n">
+      <c r="Y8" t="n">
         <v>390</v>
       </c>
-      <c r="Y8" t="n">
+      <c r="Z8" t="n">
         <v>50</v>
       </c>
-      <c r="Z8" t="n">
+      <c r="AA8" t="n">
         <v>40</v>
       </c>
-      <c r="AA8" t="n">
+      <c r="AB8" t="n">
         <v>82</v>
       </c>
-      <c r="AB8" t="n">
+      <c r="AC8" t="n">
         <v>0.16</v>
       </c>
-      <c r="AC8" t="n">
+      <c r="AD8" t="n">
         <v>620</v>
       </c>
-      <c r="AD8" t="n">
+      <c r="AE8" t="n">
         <v>0.2</v>
       </c>
-      <c r="AE8" t="n">
+      <c r="AF8" t="n">
         <v>2</v>
       </c>
-      <c r="AF8" t="n">
+      <c r="AG8" t="n">
         <v>1.4</v>
       </c>
     </row>
@@ -1518,55 +1546,58 @@
       <c r="N9" t="n">
         <v>2021</v>
       </c>
-      <c r="P9" t="n">
+      <c r="P9" s="5" t="n">
+        <v>46022</v>
+      </c>
+      <c r="Q9" t="n">
         <v>100</v>
       </c>
-      <c r="Q9" t="n">
+      <c r="R9" t="n">
         <v>0.29</v>
       </c>
-      <c r="R9" t="n">
+      <c r="S9" t="n">
         <v>30</v>
       </c>
-      <c r="S9" t="n">
+      <c r="T9" t="n">
         <v>5</v>
       </c>
-      <c r="T9" t="n">
+      <c r="U9" t="n">
         <v>150</v>
       </c>
-      <c r="U9" t="n">
+      <c r="V9" t="n">
         <v>20</v>
       </c>
-      <c r="V9" t="n">
+      <c r="W9" t="n">
         <v>85</v>
       </c>
-      <c r="W9" t="n">
+      <c r="X9" t="n">
         <v>22</v>
       </c>
-      <c r="X9" t="n">
+      <c r="Y9" t="n">
         <v>400</v>
       </c>
-      <c r="Y9" t="n">
+      <c r="Z9" t="n">
         <v>35</v>
       </c>
-      <c r="Z9" t="n">
+      <c r="AA9" t="n">
         <v>0</v>
       </c>
-      <c r="AA9" t="n">
+      <c r="AB9" t="n">
         <v>195</v>
       </c>
-      <c r="AB9" t="n">
+      <c r="AC9" t="n">
         <v>0.15</v>
       </c>
-      <c r="AC9" t="n">
+      <c r="AD9" t="n">
         <v>710</v>
       </c>
-      <c r="AD9" t="n">
+      <c r="AE9" t="n">
         <v>0.22</v>
       </c>
-      <c r="AE9" t="n">
+      <c r="AF9" t="n">
         <v>2.3</v>
       </c>
-      <c r="AF9" t="n">
+      <c r="AG9" t="n">
         <v>1.6</v>
       </c>
     </row>
@@ -1637,55 +1668,58 @@
       <c r="N10" t="n">
         <v>2022</v>
       </c>
-      <c r="P10" t="n">
+      <c r="P10" s="5" t="n">
+        <v>46022</v>
+      </c>
+      <c r="Q10" t="n">
         <v>70</v>
       </c>
-      <c r="Q10" t="n">
+      <c r="R10" t="n">
         <v>0.24</v>
       </c>
-      <c r="R10" t="n">
+      <c r="S10" t="n">
         <v>90</v>
       </c>
-      <c r="S10" t="n">
+      <c r="T10" t="n">
         <v>18</v>
       </c>
-      <c r="T10" t="n">
+      <c r="U10" t="n">
         <v>210</v>
       </c>
-      <c r="U10" t="n">
+      <c r="V10" t="n">
         <v>55</v>
       </c>
-      <c r="V10" t="n">
+      <c r="W10" t="n">
         <v>140</v>
       </c>
-      <c r="W10" t="n">
+      <c r="X10" t="n">
         <v>30</v>
       </c>
-      <c r="X10" t="n">
+      <c r="Y10" t="n">
         <v>350</v>
       </c>
-      <c r="Y10" t="n">
+      <c r="Z10" t="n">
         <v>60</v>
       </c>
-      <c r="Z10" t="n">
+      <c r="AA10" t="n">
         <v>0</v>
       </c>
-      <c r="AA10" t="n">
+      <c r="AB10" t="n">
         <v>84</v>
       </c>
-      <c r="AB10" t="n">
+      <c r="AC10" t="n">
         <v>0.12</v>
       </c>
-      <c r="AC10" t="n">
+      <c r="AD10" t="n">
         <v>710</v>
       </c>
-      <c r="AD10" t="n">
+      <c r="AE10" t="n">
         <v>0.22</v>
       </c>
-      <c r="AE10" t="n">
+      <c r="AF10" t="n">
         <v>2.3</v>
       </c>
-      <c r="AF10" t="n">
+      <c r="AG10" t="n">
         <v>1.6</v>
       </c>
     </row>
@@ -1756,55 +1790,58 @@
       <c r="N11" t="n">
         <v>2023</v>
       </c>
-      <c r="P11" t="n">
+      <c r="P11" s="5" t="n">
+        <v>46022</v>
+      </c>
+      <c r="Q11" t="n">
         <v>90</v>
       </c>
-      <c r="Q11" t="n">
+      <c r="R11" t="n">
         <v>0.37</v>
       </c>
-      <c r="R11" t="n">
+      <c r="S11" t="n">
         <v>180</v>
       </c>
-      <c r="S11" t="n">
+      <c r="T11" t="n">
         <v>32</v>
       </c>
-      <c r="T11" t="n">
+      <c r="U11" t="n">
         <v>350</v>
       </c>
-      <c r="U11" t="n">
+      <c r="V11" t="n">
         <v>90</v>
       </c>
-      <c r="V11" t="n">
+      <c r="W11" t="n">
         <v>210</v>
       </c>
-      <c r="W11" t="n">
+      <c r="X11" t="n">
         <v>38</v>
       </c>
-      <c r="X11" t="n">
+      <c r="Y11" t="n">
         <v>420</v>
       </c>
-      <c r="Y11" t="n">
+      <c r="Z11" t="n">
         <v>85</v>
       </c>
-      <c r="Z11" t="n">
+      <c r="AA11" t="n">
         <v>0</v>
       </c>
-      <c r="AA11" t="n">
+      <c r="AB11" t="n">
         <v>162</v>
       </c>
-      <c r="AB11" t="n">
+      <c r="AC11" t="n">
         <v>0.1</v>
       </c>
-      <c r="AC11" t="n">
+      <c r="AD11" t="n">
         <v>805</v>
       </c>
-      <c r="AD11" t="n">
+      <c r="AE11" t="n">
         <v>0.24</v>
       </c>
-      <c r="AE11" t="n">
+      <c r="AF11" t="n">
         <v>2.6</v>
       </c>
-      <c r="AF11" t="n">
+      <c r="AG11" t="n">
         <v>1.8</v>
       </c>
     </row>
@@ -1875,55 +1912,58 @@
       <c r="N12" t="n">
         <v>2023</v>
       </c>
-      <c r="P12" t="n">
+      <c r="P12" s="5" t="n">
+        <v>46022</v>
+      </c>
+      <c r="Q12" t="n">
         <v>80</v>
       </c>
-      <c r="Q12" t="n">
+      <c r="R12" t="n">
         <v>0.26</v>
       </c>
-      <c r="R12" t="n">
+      <c r="S12" t="n">
         <v>60</v>
       </c>
-      <c r="S12" t="n">
+      <c r="T12" t="n">
         <v>15</v>
       </c>
-      <c r="T12" t="n">
+      <c r="U12" t="n">
         <v>175</v>
       </c>
-      <c r="U12" t="n">
+      <c r="V12" t="n">
         <v>30</v>
       </c>
-      <c r="V12" t="n">
+      <c r="W12" t="n">
         <v>72</v>
       </c>
-      <c r="W12" t="n">
+      <c r="X12" t="n">
         <v>19</v>
       </c>
-      <c r="X12" t="n">
+      <c r="Y12" t="n">
         <v>220</v>
       </c>
-      <c r="Y12" t="n">
+      <c r="Z12" t="n">
         <v>28</v>
       </c>
-      <c r="Z12" t="n">
+      <c r="AA12" t="n">
         <v>0</v>
       </c>
-      <c r="AA12" t="n">
+      <c r="AB12" t="n">
         <v>104</v>
       </c>
-      <c r="AB12" t="n">
+      <c r="AC12" t="n">
         <v>0.08</v>
       </c>
-      <c r="AC12" t="n">
+      <c r="AD12" t="n">
         <v>805</v>
       </c>
-      <c r="AD12" t="n">
+      <c r="AE12" t="n">
         <v>0.24</v>
       </c>
-      <c r="AE12" t="n">
+      <c r="AF12" t="n">
         <v>2.6</v>
       </c>
-      <c r="AF12" t="n">
+      <c r="AG12" t="n">
         <v>1.8</v>
       </c>
     </row>
@@ -1994,52 +2034,55 @@
       <c r="N13" t="n">
         <v>2024</v>
       </c>
-      <c r="P13" t="n">
+      <c r="P13" s="5" t="n">
+        <v>46022</v>
+      </c>
+      <c r="Q13" t="n">
         <v>110</v>
       </c>
-      <c r="Q13" t="n">
+      <c r="R13" t="n">
         <v>0.21</v>
       </c>
-      <c r="R13" t="n">
+      <c r="S13" t="n">
         <v>25</v>
       </c>
-      <c r="S13" t="n">
+      <c r="T13" t="n">
         <v>3</v>
       </c>
-      <c r="T13" t="n">
+      <c r="U13" t="n">
         <v>120</v>
       </c>
-      <c r="U13" t="n">
+      <c r="V13" t="n">
         <v>15</v>
       </c>
-      <c r="V13" t="n">
+      <c r="W13" t="n">
         <v>35</v>
       </c>
-      <c r="W13" t="n">
+      <c r="X13" t="n">
         <v>6</v>
       </c>
-      <c r="X13" t="n">
+      <c r="Y13" t="n">
         <v>180</v>
       </c>
-      <c r="Y13" t="n">
+      <c r="Z13" t="n">
         <v>18</v>
       </c>
-      <c r="Z13" t="n">
+      <c r="AA13" t="n">
         <v>0</v>
       </c>
-      <c r="AA13" t="n">
+      <c r="AB13" t="n">
         <v>176</v>
       </c>
-      <c r="AC13" t="n">
+      <c r="AD13" t="n">
         <v>805</v>
       </c>
-      <c r="AD13" t="n">
+      <c r="AE13" t="n">
         <v>0.24</v>
       </c>
-      <c r="AE13" t="n">
+      <c r="AF13" t="n">
         <v>2.6</v>
       </c>
-      <c r="AF13" t="n">
+      <c r="AG13" t="n">
         <v>1.8</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Enable multi-firm uploads in one deals workbook
</commit_message>
<xml_diff>
--- a/PE_Fund_Data_Template.xlsx
+++ b/PE_Fund_Data_Template.xlsx
@@ -2097,36 +2097,41 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>Firm Name</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
           <t>Company Name</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Fund</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Event Date</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Event Type</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Amount</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -2135,28 +2140,33 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>Example Firm</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
           <t>Cardinal Commerce</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>Fund VII</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>2013-03-31</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>Capital Call</t>
         </is>
       </c>
-      <c r="E2" t="n">
+      <c r="F2" t="n">
         <v>-5</v>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>Initial draw</t>
         </is>
@@ -2173,56 +2183,61 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>Firm Name</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
           <t>Company Name</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Fund</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Quarter End</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Revenue</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>EBITDA</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Enterprise Value</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Net Debt</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Equity Value</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Valuation Basis</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
@@ -2231,40 +2246,45 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>Example Firm</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
           <t>Cardinal Commerce</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>Fund VII</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>2014-12-31</t>
         </is>
       </c>
-      <c r="D2" t="n">
+      <c r="E2" t="n">
         <v>72</v>
       </c>
-      <c r="E2" t="n">
+      <c r="F2" t="n">
         <v>14.5</v>
       </c>
-      <c r="F2" t="n">
+      <c r="G2" t="n">
         <v>155</v>
       </c>
-      <c r="G2" t="n">
+      <c r="H2" t="n">
         <v>40</v>
       </c>
-      <c r="H2" t="n">
+      <c r="I2" t="n">
         <v>115</v>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>Quarterly Mark</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>Finance Team</t>
         </is>
@@ -2281,41 +2301,46 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>Firm Name</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
           <t>Fund</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Quarter End</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Committed Capital</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Paid In Capital</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Distributed Capital</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>NAV</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Unfunded Commitment</t>
         </is>
@@ -2324,27 +2349,32 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>Example Firm</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
           <t>Fund VII</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>2016-12-31</t>
         </is>
       </c>
-      <c r="C2" t="n">
+      <c r="D2" t="n">
         <v>353</v>
       </c>
-      <c r="D2" t="n">
+      <c r="E2" t="n">
         <v>278.3</v>
       </c>
-      <c r="E2" t="n">
+      <c r="F2" t="n">
         <v>1078.9</v>
       </c>
-      <c r="F2" t="n">
+      <c r="G2" t="n">
         <v>0</v>
       </c>
-      <c r="G2" t="n">
+      <c r="H2" t="n">
         <v>74.7</v>
       </c>
     </row>
@@ -2359,51 +2389,56 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:J2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>Firm Name</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
           <t>Company Name</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Fund</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Baseline Date</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Target IRR</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Target MOIC</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Target Hold Years</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Target Exit Multiple</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Target Revenue CAGR</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Target EBITDA CAGR</t>
         </is>
@@ -2412,35 +2447,40 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>Example Firm</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
           <t>Cardinal Commerce</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>Fund VII</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>2012-12-01</t>
         </is>
       </c>
-      <c r="D2" t="n">
+      <c r="E2" t="n">
         <v>0.25</v>
       </c>
-      <c r="E2" t="n">
+      <c r="F2" t="n">
         <v>2.8</v>
       </c>
-      <c r="F2" t="n">
+      <c r="G2" t="n">
         <v>4.5</v>
       </c>
-      <c r="G2" t="n">
+      <c r="H2" t="n">
         <v>11.5</v>
       </c>
-      <c r="H2" t="n">
+      <c r="I2" t="n">
         <v>0.08</v>
       </c>
-      <c r="I2" t="n">
+      <c r="J2" t="n">
         <v>0.1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add organic vs acquired growth analysis page
Add 3 new Deal model fields (acquired_revenue, acquired_ebitda, acquired_tev)
for bolt-on acquisition tracking. Organic growth is derived automatically as
exit total minus entry base minus acquired contribution.

- Data layer: model columns, parser aliases, migration, Excel template
- Calculations: organic/acquired decomposition, organic CAGR, data completeness indicator
- Analysis module: summary cards, per-deal tables, Chart.js stacked bars, bridge decomposition
- Bridge integration: splits revenue driver into organic vs acquired using acquired_ebitda * x0
- Empty state with template download when no acquired data uploaded
- 21 new tests covering derivation, CAGR, edge cases, bridge reconciliation

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PE_Fund_Data_Template.xlsx
+++ b/PE_Fund_Data_Template.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AG13"/>
+  <dimension ref="A1:AJ13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -573,35 +573,50 @@
       </c>
       <c r="AA1" t="inlineStr">
         <is>
+          <t>Acquired Revenue</t>
+        </is>
+      </c>
+      <c r="AB1" t="inlineStr">
+        <is>
+          <t>Acquired EBITDA</t>
+        </is>
+      </c>
+      <c r="AC1" t="inlineStr">
+        <is>
+          <t>Acquired TEV</t>
+        </is>
+      </c>
+      <c r="AD1" t="inlineStr">
+        <is>
           <t>Realized Value</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>Unrealized Value</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>IRR</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>Fund Size</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
         <is>
           <t>Net IRR</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AI1" t="inlineStr">
         <is>
           <t>Net MOIC</t>
         </is>
       </c>
-      <c r="AG1" t="inlineStr">
+      <c r="AJ1" t="inlineStr">
         <is>
           <t>DPI</t>
         </is>
@@ -710,25 +725,25 @@
       <c r="Z2" t="n">
         <v>95</v>
       </c>
-      <c r="AA2" t="n">
+      <c r="AD2" t="n">
         <v>170</v>
       </c>
-      <c r="AB2" t="n">
+      <c r="AE2" t="n">
         <v>0</v>
       </c>
-      <c r="AC2" t="n">
+      <c r="AF2" t="n">
         <v>0.28</v>
       </c>
-      <c r="AD2" t="n">
+      <c r="AG2" t="n">
         <v>620</v>
       </c>
-      <c r="AE2" t="n">
+      <c r="AH2" t="n">
         <v>0.2</v>
       </c>
-      <c r="AF2" t="n">
+      <c r="AI2" t="n">
         <v>2</v>
       </c>
-      <c r="AG2" t="n">
+      <c r="AJ2" t="n">
         <v>1.4</v>
       </c>
     </row>
@@ -835,25 +850,25 @@
       <c r="Z3" t="n">
         <v>70</v>
       </c>
-      <c r="AA3" t="n">
+      <c r="AD3" t="n">
         <v>130</v>
       </c>
-      <c r="AB3" t="n">
+      <c r="AE3" t="n">
         <v>0</v>
       </c>
-      <c r="AC3" t="n">
+      <c r="AF3" t="n">
         <v>0.24</v>
       </c>
-      <c r="AD3" t="n">
+      <c r="AG3" t="n">
         <v>620</v>
       </c>
-      <c r="AE3" t="n">
+      <c r="AH3" t="n">
         <v>0.2</v>
       </c>
-      <c r="AF3" t="n">
+      <c r="AI3" t="n">
         <v>2</v>
       </c>
-      <c r="AG3" t="n">
+      <c r="AJ3" t="n">
         <v>1.4</v>
       </c>
     </row>
@@ -960,25 +975,25 @@
       <c r="Z4" t="n">
         <v>110</v>
       </c>
-      <c r="AA4" t="n">
+      <c r="AD4" t="n">
         <v>118</v>
       </c>
-      <c r="AB4" t="n">
+      <c r="AE4" t="n">
         <v>0</v>
       </c>
-      <c r="AC4" t="n">
+      <c r="AF4" t="n">
         <v>0.2</v>
       </c>
-      <c r="AD4" t="n">
+      <c r="AG4" t="n">
         <v>550</v>
       </c>
-      <c r="AE4" t="n">
+      <c r="AH4" t="n">
         <v>0.18</v>
       </c>
-      <c r="AF4" t="n">
+      <c r="AI4" t="n">
         <v>1.8</v>
       </c>
-      <c r="AG4" t="n">
+      <c r="AJ4" t="n">
         <v>1.2</v>
       </c>
     </row>
@@ -1085,25 +1100,25 @@
       <c r="Z5" t="n">
         <v>30</v>
       </c>
-      <c r="AA5" t="n">
+      <c r="AD5" t="n">
         <v>72</v>
       </c>
-      <c r="AB5" t="n">
+      <c r="AE5" t="n">
         <v>0</v>
       </c>
-      <c r="AC5" t="n">
+      <c r="AF5" t="n">
         <v>0.18</v>
       </c>
-      <c r="AD5" t="n">
+      <c r="AG5" t="n">
         <v>550</v>
       </c>
-      <c r="AE5" t="n">
+      <c r="AH5" t="n">
         <v>0.18</v>
       </c>
-      <c r="AF5" t="n">
+      <c r="AI5" t="n">
         <v>1.8</v>
       </c>
-      <c r="AG5" t="n">
+      <c r="AJ5" t="n">
         <v>1.2</v>
       </c>
     </row>
@@ -1210,25 +1225,25 @@
       <c r="Z6" t="n">
         <v>80</v>
       </c>
-      <c r="AA6" t="n">
+      <c r="AD6" t="n">
         <v>45</v>
       </c>
-      <c r="AB6" t="n">
+      <c r="AE6" t="n">
         <v>0</v>
       </c>
-      <c r="AC6" t="n">
+      <c r="AF6" t="n">
         <v>-0.03</v>
       </c>
-      <c r="AD6" t="n">
+      <c r="AG6" t="n">
         <v>550</v>
       </c>
-      <c r="AE6" t="n">
+      <c r="AH6" t="n">
         <v>0.18</v>
       </c>
-      <c r="AF6" t="n">
+      <c r="AI6" t="n">
         <v>1.8</v>
       </c>
-      <c r="AG6" t="n">
+      <c r="AJ6" t="n">
         <v>1.2</v>
       </c>
     </row>
@@ -1335,25 +1350,25 @@
       <c r="Z7" t="n">
         <v>55</v>
       </c>
-      <c r="AA7" t="n">
+      <c r="AD7" t="n">
         <v>90</v>
       </c>
-      <c r="AB7" t="n">
+      <c r="AE7" t="n">
         <v>75</v>
       </c>
-      <c r="AC7" t="n">
+      <c r="AF7" t="n">
         <v>0.3</v>
       </c>
-      <c r="AD7" t="n">
+      <c r="AG7" t="n">
         <v>710</v>
       </c>
-      <c r="AE7" t="n">
+      <c r="AH7" t="n">
         <v>0.22</v>
       </c>
-      <c r="AF7" t="n">
+      <c r="AI7" t="n">
         <v>2.3</v>
       </c>
-      <c r="AG7" t="n">
+      <c r="AJ7" t="n">
         <v>1.6</v>
       </c>
     </row>
@@ -1457,25 +1472,25 @@
       <c r="Z8" t="n">
         <v>50</v>
       </c>
-      <c r="AA8" t="n">
+      <c r="AD8" t="n">
         <v>40</v>
       </c>
-      <c r="AB8" t="n">
+      <c r="AE8" t="n">
         <v>82</v>
       </c>
-      <c r="AC8" t="n">
+      <c r="AF8" t="n">
         <v>0.16</v>
       </c>
-      <c r="AD8" t="n">
+      <c r="AG8" t="n">
         <v>620</v>
       </c>
-      <c r="AE8" t="n">
+      <c r="AH8" t="n">
         <v>0.2</v>
       </c>
-      <c r="AF8" t="n">
+      <c r="AI8" t="n">
         <v>2</v>
       </c>
-      <c r="AG8" t="n">
+      <c r="AJ8" t="n">
         <v>1.4</v>
       </c>
     </row>
@@ -1579,25 +1594,25 @@
       <c r="Z9" t="n">
         <v>35</v>
       </c>
-      <c r="AA9" t="n">
+      <c r="AD9" t="n">
         <v>0</v>
       </c>
-      <c r="AB9" t="n">
+      <c r="AE9" t="n">
         <v>195</v>
       </c>
-      <c r="AC9" t="n">
+      <c r="AF9" t="n">
         <v>0.15</v>
       </c>
-      <c r="AD9" t="n">
+      <c r="AG9" t="n">
         <v>710</v>
       </c>
-      <c r="AE9" t="n">
+      <c r="AH9" t="n">
         <v>0.22</v>
       </c>
-      <c r="AF9" t="n">
+      <c r="AI9" t="n">
         <v>2.3</v>
       </c>
-      <c r="AG9" t="n">
+      <c r="AJ9" t="n">
         <v>1.6</v>
       </c>
     </row>
@@ -1701,25 +1716,25 @@
       <c r="Z10" t="n">
         <v>60</v>
       </c>
-      <c r="AA10" t="n">
+      <c r="AD10" t="n">
         <v>0</v>
       </c>
-      <c r="AB10" t="n">
+      <c r="AE10" t="n">
         <v>84</v>
       </c>
-      <c r="AC10" t="n">
+      <c r="AF10" t="n">
         <v>0.12</v>
       </c>
-      <c r="AD10" t="n">
+      <c r="AG10" t="n">
         <v>710</v>
       </c>
-      <c r="AE10" t="n">
+      <c r="AH10" t="n">
         <v>0.22</v>
       </c>
-      <c r="AF10" t="n">
+      <c r="AI10" t="n">
         <v>2.3</v>
       </c>
-      <c r="AG10" t="n">
+      <c r="AJ10" t="n">
         <v>1.6</v>
       </c>
     </row>
@@ -1823,25 +1838,25 @@
       <c r="Z11" t="n">
         <v>85</v>
       </c>
-      <c r="AA11" t="n">
+      <c r="AD11" t="n">
         <v>0</v>
       </c>
-      <c r="AB11" t="n">
+      <c r="AE11" t="n">
         <v>162</v>
       </c>
-      <c r="AC11" t="n">
+      <c r="AF11" t="n">
         <v>0.1</v>
       </c>
-      <c r="AD11" t="n">
+      <c r="AG11" t="n">
         <v>805</v>
       </c>
-      <c r="AE11" t="n">
+      <c r="AH11" t="n">
         <v>0.24</v>
       </c>
-      <c r="AF11" t="n">
+      <c r="AI11" t="n">
         <v>2.6</v>
       </c>
-      <c r="AG11" t="n">
+      <c r="AJ11" t="n">
         <v>1.8</v>
       </c>
     </row>
@@ -1945,25 +1960,25 @@
       <c r="Z12" t="n">
         <v>28</v>
       </c>
-      <c r="AA12" t="n">
+      <c r="AD12" t="n">
         <v>0</v>
       </c>
-      <c r="AB12" t="n">
+      <c r="AE12" t="n">
         <v>104</v>
       </c>
-      <c r="AC12" t="n">
+      <c r="AF12" t="n">
         <v>0.08</v>
       </c>
-      <c r="AD12" t="n">
+      <c r="AG12" t="n">
         <v>805</v>
       </c>
-      <c r="AE12" t="n">
+      <c r="AH12" t="n">
         <v>0.24</v>
       </c>
-      <c r="AF12" t="n">
+      <c r="AI12" t="n">
         <v>2.6</v>
       </c>
-      <c r="AG12" t="n">
+      <c r="AJ12" t="n">
         <v>1.8</v>
       </c>
     </row>
@@ -2067,22 +2082,22 @@
       <c r="Z13" t="n">
         <v>18</v>
       </c>
-      <c r="AA13" t="n">
+      <c r="AD13" t="n">
         <v>0</v>
       </c>
-      <c r="AB13" t="n">
+      <c r="AE13" t="n">
         <v>176</v>
       </c>
-      <c r="AD13" t="n">
+      <c r="AG13" t="n">
         <v>805</v>
       </c>
-      <c r="AE13" t="n">
+      <c r="AH13" t="n">
         <v>0.24</v>
       </c>
-      <c r="AF13" t="n">
+      <c r="AI13" t="n">
         <v>2.6</v>
       </c>
-      <c r="AG13" t="n">
+      <c r="AJ13" t="n">
         <v>1.8</v>
       </c>
     </row>

</xml_diff>